<commit_message>
Use distinct itinerary day photos
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -599,12 +599,12 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>/itinerary/cover-australia-editorial.png</t>
+          <t>/itinerary/d0-shanghai-departure.png</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>澳洲十六日旅行封面</t>
+          <t>上海机场夜间出发</t>
         </is>
       </c>
     </row>
@@ -735,12 +735,12 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>/itinerary/melbourne-city-morning.png</t>
+          <t>/itinerary/d2-melbourne-laneways-market.png</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>墨尔本城市与咖啡文化</t>
+          <t>墨尔本巷弄与市集</t>
         </is>
       </c>
     </row>
@@ -871,12 +871,12 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>/itinerary/great-ocean-road-coast.png</t>
+          <t>/itinerary/d4-twelve-apostles-gorge.png</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>大洋路悬崖与海蚀柱</t>
+          <t>十二使徒岩与峡谷海岸</t>
         </is>
       </c>
     </row>
@@ -939,12 +939,12 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>/itinerary/great-ocean-road-coast.png</t>
+          <t>/itinerary/d5-port-campbell-morning.png</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>大洋路清晨海岸</t>
+          <t>Port Campbell 清晨海岸</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1075,12 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>/itinerary/cairns-reef-lagoon.png</t>
+          <t>/itinerary/d7-great-barrier-reef-pontoon.png</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>大堡礁热带海水与珊瑚</t>
+          <t>大堡礁外礁平台</t>
         </is>
       </c>
     </row>
@@ -1211,12 +1211,12 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>/itinerary/daintree-rainforest.png</t>
+          <t>/itinerary/d9-atherton-tablelands-waterfall.png</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>热带雨林与高原瀑布氛围</t>
+          <t>阿瑟顿高原瀑布</t>
         </is>
       </c>
     </row>
@@ -1279,12 +1279,12 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>/itinerary/cairns-reef-lagoon.png</t>
+          <t>/itinerary/d10-cairns-rustys-market.png</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>凯恩斯海滨与泻湖</t>
+          <t>凯恩斯市场与海滨</t>
         </is>
       </c>
     </row>
@@ -1347,12 +1347,12 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>/itinerary/sydney-harbor-evening.png</t>
+          <t>/itinerary/d11-sydney-arrival-rocks.png</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>悉尼海港夜景</t>
+          <t>悉尼 The Rocks 夜景</t>
         </is>
       </c>
     </row>
@@ -1415,12 +1415,12 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>/itinerary/sydney-harbor-evening.png</t>
+          <t>/itinerary/d12-sydney-opera-garden.png</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>悉尼歌剧院与海港桥</t>
+          <t>悉尼歌剧院与植物园</t>
         </is>
       </c>
     </row>
@@ -1483,12 +1483,12 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>/itinerary/sydney-harbor-evening.png</t>
+          <t>/itinerary/d13-blue-mountains-seacliff-choice.png</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>悉尼周边自然一日游</t>
+          <t>蓝山与南海岸弹性路线</t>
         </is>
       </c>
     </row>
@@ -1551,12 +1551,12 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>/itinerary/sydney-harbor-evening.png</t>
+          <t>/itinerary/d14-whale-bondi-coast.png</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>悉尼海港与海岸</t>
+          <t>悉尼观鲸与 Bondi 海岸</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>/itinerary/cover-australia-editorial.png</t>
+          <t>/itinerary/d16-return-flight.png</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add daily meal map to itinerary
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -1708,7 +1708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:H110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5259,27 +5259,27 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Bondi / CBD</t>
+          <t>Totti’s Bondi / Icebergs / Bondi Bistro</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>晚餐</t>
+          <t>晚餐（Totti’s 放 D14，Bondi 动线顺）</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>轻松收尾</t>
+          <t>Bondi 晚餐核心日</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>看体力决定回市区还是海边吃</t>
+          <t>优先 Totti’s Bondi；Icebergs / Bondi Bistro 备选，Chickorea 可作午餐备选</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>bondi-bistro-map</t>
+          <t>tottis-bondi-map,tottis-bondi-official,icebergs-map,bondi-bistro-map,chickorea-map</t>
         </is>
       </c>
     </row>
@@ -5482,6 +5482,642 @@
           <t>sydney-airport-map,trs-official</t>
         </is>
       </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>d1</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>900</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>早餐：CBD café / Operator25（可选 Brunch）；午餐：酒店简餐 / Pho Tùng（可选）；晚餐：Southbank Riverland</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Southbank Riverland</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>轻恢复</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>operator25-map,pho-tung-map,riverland-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>d2</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>900</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>早餐：Lune Croissanterie / Operator25 Brunch；午餐：Degraves / Hardware Lane / Market Lane Coffee；晚餐：Supernormal / Palermo（可选升级）</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Supernormal / Palermo（可选升级）</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>QVM hot jam donut + American Doughnut Kitchen 必吃</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>lune-map,operator25-map,market-lane-coffee-map,american-doughnut-map,supernormal-map,palermo-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>d3</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>900</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>早餐：出发咖啡；午餐：Lorne café / Snow Monkey Ramen（备选）；晚餐：Apollo Bay Fishermen’s Co-op / seafood café</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Apollo Bay Fishermen’s Co-op / seafood café</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>fish &amp; chips 必吃</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>snow-monkey-ramen-map,fishermens-coop-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>d4</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>900</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>早餐：Apollo Bay café；午餐：轻食 / picnic；晚餐：12 Rocks Café / George’s / BBQ（若住宿确认）</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>12 Rocks Café / George’s / BBQ（若住宿确认）</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>控制饮食</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>twelve-rocks-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>d5</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>900</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>早餐：Port Campbell café；午餐：Colac / Timboon Ice Cream（🔥）；晚餐：机场酒店简餐</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>机场酒店简餐</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>冰淇淋补偿日</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>timboon-icecream-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>d6</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>900</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>早餐：飞机 / 机场；午餐：简餐 / Overlay Coffee（花生拿铁🔥）；晚餐：Night Market</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Night Market</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>花生咖啡可试</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>overlay-coffee-map,cairns-night-market-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>d7</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>900</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>早餐：酒店轻食；午餐：Reef Magic 船上自助；晚餐：Prawn Star / Salt House</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Prawn Star / Salt House</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>海鲜核心日</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>prawn-star-map,salt-house-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>d8</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>900</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>早餐：酒店早餐；午餐：团餐；晚餐：凯恩斯随便</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>凯恩斯随便</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Daintree Ice Cream 必吃</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>daintree-icecream-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>d9</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>900</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>早餐：café 早餐；午餐：Gallo Dairyland / Millaa Millaa；晚餐：回凯恩斯随便</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>回凯恩斯随便</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>奶制品 + 瀑布</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>gallo-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>d10</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>900</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>早餐：Rusty’s Market / Market 水果；午餐：简餐；晚餐：Prawn Star / seafood café（优先）</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Prawn Star / seafood café（优先）</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>修复 + 海鲜</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>prawn-star-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>d11</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>900</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>早餐：café / A.P Bakery（可选）；午餐：飞机 / 机场 / mezze feast；晚餐：The Rocks pub</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>The Rocks pub</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>转场</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>ap-bakery-map,the-rocks-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>d12</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>900</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>早餐：bills / Toby’s Estate；午餐：Sydney Fish Market / Gumshara / Mamak；晚餐：Hello Auntie</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Hello Auntie</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>城市核心日</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>bills-sydney-map,tobys-estate-map,sydney-fish-market-map,gumshara-map,mamak-map,hello-auntie-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>d13</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>900</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>早餐：café；午餐：Leura / Kiama Hungry Monkey（🔥）；晚餐：CBD 简餐 / Bar Totti’s CBD</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>CBD 简餐 / Bar Totti’s CBD</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>机动日</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>kiama-hungry-monkey-map,bar-tottis-cbd-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>d14</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>900</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>早餐：CBD café；午餐：Bondi casual / Chickorea（备选）；晚餐：Totti’s Bondi / Icebergs / Bondi Bistro（🔥）</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Totti’s Bondi / Icebergs / Bondi Bistro（🔥）</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>最适合放 Totti’s 的一天；Bondi 动线顺</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>chickorea-map,tottis-bondi-map,tottis-bondi-official,icebergs-map,bondi-bistro-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>d15</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>900</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>早餐：café / Single O / Toby’s Estate；午餐：Manly fish &amp; chips / Hugos / Felons Manly；晚餐：Cafe Sydney（终极🔥）</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Cafe Sydney（终极🔥）</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>收尾夜</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>single-o-map,tobys-estate-map,hugos-manly-map,felons-manly-map,cafe-sydney-map,cafe-sydney-official</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>d16</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>900</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>饮食安排</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>早餐：机场早餐；午餐：飞机；晚餐：无</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>结束</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H94"/>
@@ -5495,7 +6131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G103"/>
+  <dimension ref="A1:G113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -8499,6 +9135,296 @@
       <c r="G103" s="2" t="inlineStr">
         <is>
           <t>Google Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>lune-map</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Lune Croissanterie</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Lune+Croissanterie+Melbourne</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>market-lane-coffee-map</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Market Lane Coffee</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Market+Lane+Coffee+Melbourne</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>pho-tung-map</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Pho Tùng Melbourne</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Pho+Tung+Melbourne</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>snow-monkey-ramen-map</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Snow Monkey Ramen Lorne</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Snow+Monkey+Ramen+Lorne</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>timboon-icecream-map</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Timboon Fine Ice Cream</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Timboon+Fine+Ice+Cream</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>overlay-coffee-map</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Overlay Coffee Cairns</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Overlay+Coffee+Cairns</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>bills-sydney-map</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>bills Sydney</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=bills+Sydney</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>bar-tottis-cbd-map</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Bar Totti's CBD</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Bar+Totti%27s+Sydney+CBD</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>tottis-bondi-map</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Totti's Bondi</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Totti%27s+Bondi</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>tottis-bondi-official</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Totti's Bondi</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://merivale.com/venues/tottis/</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>官网</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refine itinerary hero and D3 image
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -803,12 +803,12 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>/itinerary/great-ocean-road-coast.png</t>
+          <t>/itinerary/d3-great-ocean-road-lorne.png</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>大洋路海岸线</t>
+          <t>大洋路早段海岸公路与灯塔</t>
         </is>
       </c>
     </row>
@@ -6117,7 +6117,6 @@
           <t>结束</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H94"/>
@@ -9159,8 +9158,6 @@
           <t>https://www.google.com/maps/search/?api=1&amp;query=Lune+Croissanterie+Melbourne</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
-      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
           <t>Google Maps</t>
@@ -9188,8 +9185,6 @@
           <t>https://www.google.com/maps/search/?api=1&amp;query=Market+Lane+Coffee+Melbourne</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
-      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
           <t>Google Maps</t>
@@ -9217,8 +9212,6 @@
           <t>https://www.google.com/maps/search/?api=1&amp;query=Pho+Tung+Melbourne</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
-      <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
           <t>Google Maps</t>
@@ -9246,8 +9239,6 @@
           <t>https://www.google.com/maps/search/?api=1&amp;query=Snow+Monkey+Ramen+Lorne</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
-      <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
           <t>Google Maps</t>
@@ -9275,8 +9266,6 @@
           <t>https://www.google.com/maps/search/?api=1&amp;query=Timboon+Fine+Ice+Cream</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
-      <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
           <t>Google Maps</t>
@@ -9304,8 +9293,6 @@
           <t>https://www.google.com/maps/search/?api=1&amp;query=Overlay+Coffee+Cairns</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
           <t>Google Maps</t>
@@ -9333,8 +9320,6 @@
           <t>https://www.google.com/maps/search/?api=1&amp;query=bills+Sydney</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
-      <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
           <t>Google Maps</t>
@@ -9362,8 +9347,6 @@
           <t>https://www.google.com/maps/search/?api=1&amp;query=Bar+Totti%27s+Sydney+CBD</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
           <t>Google Maps</t>
@@ -9391,8 +9374,6 @@
           <t>https://www.google.com/maps/search/?api=1&amp;query=Totti%27s+Bondi</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
-      <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
           <t>Google Maps</t>
@@ -9420,8 +9401,6 @@
           <t>https://merivale.com/venues/tottis/</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
           <t>官网</t>

</xml_diff>

<commit_message>
feat: replace D15 Manly plan with Taronga Zoo
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R0e845cbed237445b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R9eb4f1820f9541ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R5d7f9a15295247e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R7978bb33877f467a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R2fa8040d35dc49e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R2e5ee33424a04ae1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R446f649a378f482e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R20bdbe3ba2b2413a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R4b0da47c308440f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R04738e3f54ee47d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R8ae9fe880a1444f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R163255b5ce384fda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R3366935c4240479b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R3398de61b0564ae9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R6933ad6862944364"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R867aec21b6f34b97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="Ra1f5b7fe54a844e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="Re095f495fa3d4d45"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1878,55 +1878,41 @@
       <x:c r="G17" t="n">
         <x:v>151.2093</x:v>
       </x:c>
-      <x:c r="H17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Manly Ferry + 最后采购 + Cafe Sydney</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Manly Ferry + Manly Beach + QVB / Chemist Warehouse 最后采购 + Cafe Sydney 17:30 Outdoor Terrace Dining 告别晚餐已订</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Oaks Sydney Goldsbrough Suites</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悉尼早晚凉，渡轮上海风明显。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">薄外套随身；晚餐注意 smart dress code。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/sydney-harbor-evening.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悉尼海港黄昏</x:t>
-        </x:is>
+      <x:c r="H17" t="str">
+        <x:v>Taronga Zoo + 最后采购 + Cafe Sydney</x:v>
+      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>Taronga Zoo + Sydney Harbour Ferry + QVB / Chemist Warehouse 最后采购 + Cafe Sydney 17:30 Outdoor Terrace Dining 告别晚餐已订</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>Oaks Sydney Goldsbrough Suites</x:v>
+      </x:c>
+      <x:c r="K17" t="str">
+        <x:v>悉尼早晚凉，渡轮甲板和动物园高处有风。</x:v>
+      </x:c>
+      <x:c r="L17" t="str">
+        <x:v>薄外套随身；动物园步行较多，穿舒适鞋；晚餐注意 smart casual。</x:v>
+      </x:c>
+      <x:c r="M17" t="str">
+        <x:v>/itinerary/d15-taronga-zoo-harbour.png</x:v>
+      </x:c>
+      <x:c r="N17" t="str">
+        <x:v>Taronga Zoo 长颈鹿与悉尼港景观</x:v>
       </x:c>
       <x:c r="O17" s="8" t="str">
-        <x:v>Ferry + 步行 / 市内交通</x:v>
+        <x:v>F2 Ferry + 步行 / 市内交通</x:v>
       </x:c>
       <x:c r="P17" s="8" t="str">
-        <x:v>上午按渡轮班次出发；16:40 左右前往 Circular Quay</x:v>
+        <x:v>08:30 左右出门前往 Circular Quay；16:40 前往 Cafe Sydney</x:v>
       </x:c>
       <x:c r="Q17" s="8" t="str">
         <x:v>oaks-sydney-map</x:v>
       </x:c>
       <x:c r="R17" s="8" t="str">
-        <x:v>manly-ferry-map</x:v>
+        <x:v>taronga-zoo-map</x:v>
       </x:c>
       <x:c r="S17" s="8" t="str">
-        <x:v>no-fixed-ticket</x:v>
+        <x:v>taronga-zoo-official</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -6844,439 +6830,340 @@
       </x:c>
     </x:row>
     <x:row r="123">
-      <x:c r="A123" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d15</x:t>
-        </x:is>
+      <x:c r="A123" t="str">
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B123" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C123" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">上午</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D123" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Circular Quay → Manly</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E123" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">坐公共 Manly Ferry 去 Manly</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F123" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">渡轮本身就是海港巡游</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G123" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">不需要额外订 Captain Cook 观光船；公共 F1 Manly Ferry 已经很经典</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H123" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">circular-quay-map,manly-ferry-map</x:t>
-        </x:is>
+      <x:c r="C123" t="str">
+        <x:v>08:30–09:00</x:v>
+      </x:c>
+      <x:c r="D123" t="str">
+        <x:v>酒店 → Circular Quay</x:v>
+      </x:c>
+      <x:c r="E123" t="str">
+        <x:v>前往 Taronga Zoo Ferry 码头</x:v>
+      </x:c>
+      <x:c r="F123" t="str">
+        <x:v>悉尼最后一天慢启动</x:v>
+      </x:c>
+      <x:c r="G123" t="str">
+        <x:v>提前查看 F2 渡轮班次，建议到 Circular Quay Wharf 4</x:v>
+      </x:c>
+      <x:c r="H123" t="str">
+        <x:v>oaks-sydney-map,circular-quay-map,taronga-ferry-official</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
-      <x:c r="A124" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d15</x:t>
-        </x:is>
+      <x:c r="A124" t="str">
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B124" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="C124" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">中午</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D124" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Manly Beach</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E124" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">海边午餐、散步</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F124" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">比 Bondi 更松弛</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G124" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">可吃 fish &amp; chips / beach brunch，不要吃太撑</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H124" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">manly-beach-map,hugos-manly-map,felons-manly-map</x:t>
-        </x:is>
+      <x:c r="C124" t="str">
+        <x:v>09:15–10:00</x:v>
+      </x:c>
+      <x:c r="D124" t="str">
+        <x:v>Circular Quay → Taronga Zoo Wharf</x:v>
+      </x:c>
+      <x:c r="E124" t="str">
+        <x:v>搭乘 F2 Ferry 前往 Taronga Zoo</x:v>
+      </x:c>
+      <x:c r="F124" t="str">
+        <x:v>Opera House + Harbour Bridge + Skyline</x:v>
+      </x:c>
+      <x:c r="G124" t="str">
+        <x:v>建议坐上层甲板；渡轮是今天的重要体验，不只是交通</x:v>
+      </x:c>
+      <x:c r="H124" t="str">
+        <x:v>circular-quay-map,taronga-ferry-official,taronga-zoo-map</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
-      <x:c r="A125" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d15</x:t>
-        </x:is>
+      <x:c r="A125" t="str">
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B125" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="C125" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14:30–15:30</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D125" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">QVB / Chemist Warehouse / 超市</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E125" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">最后采购</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F125" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">药妆、保健品、伴手礼</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G125" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">今天必须买完；注意同店 A$300 以上 TRS 退税条件</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H125" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">qvb-map,chemist-warehouse-map</x:t>
-        </x:is>
+      <x:c r="C125" t="str">
+        <x:v>10:00–13:30</x:v>
+      </x:c>
+      <x:c r="D125" t="str">
+        <x:v>Taronga Zoo</x:v>
+      </x:c>
+      <x:c r="E125" t="str">
+        <x:v>游览动物园，优先 Australian Wildlife 区域</x:v>
+      </x:c>
+      <x:c r="F125" t="str">
+        <x:v>Koala / Kangaroo / Wallaby / Wombat + 悉尼港景观</x:v>
+      </x:c>
+      <x:c r="G125" t="str">
+        <x:v>不追求全部动物；当天 keeper talk 以官网和现场时间为准</x:v>
+      </x:c>
+      <x:c r="H125" t="str">
+        <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
-      <x:c r="A126" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d15</x:t>
-        </x:is>
+      <x:c r="A126" t="str">
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B126" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="C126" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15:30–16:30</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D126" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">酒店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E126" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">整理购物袋和退税物品</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F126" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">为 D16 机场退税做准备</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G126" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">把 tax invoice、商品、护照、支付卡放好；行李别乱</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H126" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">oaks-sydney-map,trs-official</x:t>
-        </x:is>
+      <x:c r="C126" t="str">
+        <x:v>13:30–14:00</x:v>
+      </x:c>
+      <x:c r="D126" t="str">
+        <x:v>Taronga Zoo Wharf → Circular Quay</x:v>
+      </x:c>
+      <x:c r="E126" t="str">
+        <x:v>搭乘 F2 Ferry 返回市区</x:v>
+      </x:c>
+      <x:c r="F126" t="str">
+        <x:v>再看一次悉尼港</x:v>
+      </x:c>
+      <x:c r="G126" t="str">
+        <x:v>回程可休息，给下午采购和晚餐留体力</x:v>
+      </x:c>
+      <x:c r="H126" t="str">
+        <x:v>taronga-zoo-map,taronga-ferry-official,circular-quay-map</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
-      <x:c r="A127" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d15</x:t>
-        </x:is>
+      <x:c r="A127" t="str">
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B127" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="C127" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16:40</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D127" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">酒店 → Circular Quay</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E127" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">出发去 Cafe Sydney</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F127" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">避免迟到</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G127" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">穿得稍正式，但带外套，Outdoor Terrace 晚上可能冷</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H127" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:t>
-        </x:is>
+      <x:c r="C127" t="str">
+        <x:v>14:00–15:30</x:v>
+      </x:c>
+      <x:c r="D127" t="str">
+        <x:v>QVB / Chemist Warehouse / CBD</x:v>
+      </x:c>
+      <x:c r="E127" t="str">
+        <x:v>最后采购</x:v>
+      </x:c>
+      <x:c r="F127" t="str">
+        <x:v>药妆、保健品、伴手礼</x:v>
+      </x:c>
+      <x:c r="G127" t="str">
+        <x:v>今天完成所有购物；保留 tax invoice 并核对 TRS 条件</x:v>
+      </x:c>
+      <x:c r="H127" t="str">
+        <x:v>qvb-map,chemist-warehouse-map</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
-      <x:c r="A128" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d15</x:t>
-        </x:is>
+      <x:c r="A128" t="str">
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B128" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="C128" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">17:00–17:20</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D128" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Circular Quay 外部</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E128" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">外面拍日落 / 蓝调光线</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F128" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">歌剧院、海港桥、夕光</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G128" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">不要 17:30 才从酒店出发</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H128" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">circular-quay-map,opera-house-map</x:t>
-        </x:is>
+      <x:c r="C128" t="str">
+        <x:v>15:30–16:20</x:v>
+      </x:c>
+      <x:c r="D128" t="str">
+        <x:v>酒店</x:v>
+      </x:c>
+      <x:c r="E128" t="str">
+        <x:v>整理 TRS 和返程行李</x:v>
+      </x:c>
+      <x:c r="F128" t="str">
+        <x:v>为 D16 返程准备</x:v>
+      </x:c>
+      <x:c r="G128" t="str">
+        <x:v>发票、商品、护照和支付卡集中整理</x:v>
+      </x:c>
+      <x:c r="H128" t="str">
+        <x:v>oaks-sydney-map,trs-official</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
-      <x:c r="A129" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d15</x:t>
-        </x:is>
+      <x:c r="A129" t="str">
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B129" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="C129" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">17:30</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D129" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cafe Sydney</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E129" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Outdoor Terrace Dining 告别晚餐已订</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F129" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">海港景观 + seafood / modern Australian</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G129" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">香槟 add-on 不需要，到店后再点酒更灵活；注意 1.5% card surcharge</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H129" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">cafe-sydney-map,cafe-sydney-official</x:t>
-        </x:is>
+      <x:c r="C129" t="str">
+        <x:v>16:40</x:v>
+      </x:c>
+      <x:c r="D129" t="str">
+        <x:v>酒店 → Circular Quay</x:v>
+      </x:c>
+      <x:c r="E129" t="str">
+        <x:v>前往 Cafe Sydney</x:v>
+      </x:c>
+      <x:c r="F129" t="str">
+        <x:v>避免迟到</x:v>
+      </x:c>
+      <x:c r="G129" t="str">
+        <x:v>换 smart casual；Outdoor Terrace 注意带外套</x:v>
+      </x:c>
+      <x:c r="H129" t="str">
+        <x:v>oaks-sydney-map,circular-quay-map,cafe-sydney-map</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
-      <x:c r="A130" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d15</x:t>
-        </x:is>
+      <x:c r="A130" t="str">
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B130" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="C130" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">晚上</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D130" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Circular Quay / 酒店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E130" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">晚餐后回酒店</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F130" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">全程收尾</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G130" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">回去后最终整理 D16 返程行李</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H130" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">circular-quay-map,oaks-sydney-map</x:t>
-        </x:is>
+      <x:c r="C130" t="str">
+        <x:v>17:00–17:15</x:v>
+      </x:c>
+      <x:c r="D130" t="str">
+        <x:v>Circular Quay</x:v>
+      </x:c>
+      <x:c r="E130" t="str">
+        <x:v>日落前拍摄</x:v>
+      </x:c>
+      <x:c r="F130" t="str">
+        <x:v>Opera House + Harbour Bridge + 蓝调前光线</x:v>
+      </x:c>
+      <x:c r="G130" t="str">
+        <x:v>不要拖到 17:30 才到附近</x:v>
+      </x:c>
+      <x:c r="H130" t="str">
+        <x:v>circular-quay-map,opera-house-map</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
-      <x:c r="A131" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d15</x:t>
-        </x:is>
+      <x:c r="A131" t="str">
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B131" t="n">
-        <x:v>900</x:v>
-      </x:c>
-      <x:c r="C131" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">饮食</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D131" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">饮食安排</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E131" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">早餐：café / Single O / Toby’s Estate；午餐：Manly fish &amp; chips / Hugos / Felons Manly；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F131" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">每日餐食参考</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G131" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16:40 左右出发去 Circular Quay；17:00–17:20 外面拍日落光线；17:30 入座；注意带外套</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H131" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">single-o-map,tobys-estate-map,manly-beach-map,hugos-manly-map,felons-manly-map,cafe-sydney-map,cafe-sydney-official</x:t>
-        </x:is>
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C131" t="str">
+        <x:v>17:30</x:v>
+      </x:c>
+      <x:c r="D131" t="str">
+        <x:v>Cafe Sydney</x:v>
+      </x:c>
+      <x:c r="E131" t="str">
+        <x:v>Outdoor Terrace Dining 告别晚餐已订</x:v>
+      </x:c>
+      <x:c r="F131" t="str">
+        <x:v>最后一晚海港晚餐</x:v>
+      </x:c>
+      <x:c r="G131" t="str">
+        <x:v>按预订时间入座；到店后再灵活点酒</x:v>
+      </x:c>
+      <x:c r="H131" t="str">
+        <x:v>cafe-sydney-map,cafe-sydney-official</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
-      <x:c r="A132" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d16</x:t>
-        </x:is>
+      <x:c r="A132" t="str">
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B132" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C132" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">上午</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D132" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悉尼机场</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E132" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">办理 TRS 退税，登机返程。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F132" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">满载而归</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G132" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">提前下载 TRS App 填好信息，可走快速通道。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H132" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">sydney-airport-map,trs-official</x:t>
-        </x:is>
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C132" t="str">
+        <x:v>晚上</x:v>
+      </x:c>
+      <x:c r="D132" t="str">
+        <x:v>酒店</x:v>
+      </x:c>
+      <x:c r="E132" t="str">
+        <x:v>最终整理</x:v>
+      </x:c>
+      <x:c r="F132" t="str">
+        <x:v>返程准备</x:v>
+      </x:c>
+      <x:c r="G132" t="str">
+        <x:v>回酒店后完成 D16 行李和退税物品检查</x:v>
+      </x:c>
+      <x:c r="H132" t="str">
+        <x:v>oaks-sydney-map,trs-official</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
-      <x:c r="A133" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d16</x:t>
-        </x:is>
+      <x:c r="A133" t="str">
+        <x:v>d15</x:v>
       </x:c>
       <x:c r="B133" t="n">
         <x:v>900</x:v>
       </x:c>
-      <x:c r="C133" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">饮食</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D133" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">饮食安排</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E133" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">早餐：机场早餐；午餐：飞机；晚餐：无</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F133" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">无</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G133" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">结束</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="C133" t="str">
+        <x:v>饮食</x:v>
+      </x:c>
+      <x:c r="D133" t="str">
+        <x:v>饮食安排</x:v>
+      </x:c>
+      <x:c r="E133" t="str">
+        <x:v>早餐：café / Single O / Toby’s Estate；午餐：Taronga Zoo Café / 自带轻食 / Circular Quay casual lunch；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+      </x:c>
+      <x:c r="F133" t="str">
+        <x:v>每日餐食参考</x:v>
+      </x:c>
+      <x:c r="G133" t="str">
+        <x:v>动物园午餐保持轻量；16:40 出发去 Circular Quay；17:00–17:15 拍日落；17:30 入座</x:v>
+      </x:c>
+      <x:c r="H133" t="str">
+        <x:v>single-o-map,tobys-estate-map,taronga-zoo-map,circular-quay-map,cafe-sydney-map,cafe-sydney-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" t="str">
+        <x:v>d16</x:v>
+      </x:c>
+      <x:c r="B134" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C134" t="str">
+        <x:v>上午</x:v>
+      </x:c>
+      <x:c r="D134" t="str">
+        <x:v>悉尼机场</x:v>
+      </x:c>
+      <x:c r="E134" t="str">
+        <x:v>办理 TRS 退税，登机返程。</x:v>
+      </x:c>
+      <x:c r="F134" t="str">
+        <x:v>满载而归</x:v>
+      </x:c>
+      <x:c r="G134" t="str">
+        <x:v>提前下载 TRS App 填好信息，可走快速通道。</x:v>
+      </x:c>
+      <x:c r="H134" t="str">
+        <x:v>sydney-airport-map,trs-official</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" t="str">
+        <x:v>d16</x:v>
+      </x:c>
+      <x:c r="B135" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="C135" t="str">
+        <x:v>饮食</x:v>
+      </x:c>
+      <x:c r="D135" t="str">
+        <x:v>饮食安排</x:v>
+      </x:c>
+      <x:c r="E135" t="str">
+        <x:v>早餐：机场早餐；午餐：飞机；晚餐：无</x:v>
+      </x:c>
+      <x:c r="F135" t="str">
+        <x:v>无</x:v>
+      </x:c>
+      <x:c r="G135" t="str">
+        <x:v>结束</x:v>
+      </x:c>
+      <x:c r="H135" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8981,30 +8868,22 @@
       </x:c>
     </x:row>
     <x:row r="63">
-      <x:c r="A63" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">manly-ferry-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B63" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Manly Ferry</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C63" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D63" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.google.com/maps/search/?api=1&amp;query=Manly+Ferry+Sydney</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G63" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Google Maps</x:t>
-        </x:is>
+      <x:c r="A63" t="str">
+        <x:v>taronga-zoo-map</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>Taronga Zoo Sydney</x:v>
+      </x:c>
+      <x:c r="C63" t="str">
+        <x:v>map</x:v>
+      </x:c>
+      <x:c r="D63" t="str">
+        <x:v>https://www.google.com/maps/search/?api=1&amp;query=Taronga+Zoo+Sydney</x:v>
+      </x:c>
+      <x:c r="E63" t="str"/>
+      <x:c r="F63" t="str"/>
+      <x:c r="G63" t="str">
+        <x:v>Google Maps</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -9764,85 +9643,49 @@
       </x:c>
     </x:row>
     <x:row r="92">
-      <x:c r="A92" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">manly-beach-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B92" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Manly Beach</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C92" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D92" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.google.com/maps/search/?api=1&amp;query=Manly+Beach+Sydney</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G92" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Google Maps</x:t>
-        </x:is>
+      <x:c r="A92" t="str">
+        <x:v>taronga-zoo-official</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>Taronga Zoo Sydney</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D92" t="str">
+        <x:v>https://www.taronga.org.au/sydney-zoo</x:v>
+      </x:c>
+      <x:c r="E92" t="str"/>
+      <x:c r="F92" t="str"/>
+      <x:c r="G92" t="str">
+        <x:v>Taronga Zoo 官网</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
-      <x:c r="A93" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">hugos-manly-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B93" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Hugos Manly</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C93" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">restaurant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D93" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.google.com/maps/search/?api=1&amp;query=Hugos+Manly</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G93" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Google Maps</x:t>
-        </x:is>
+      <x:c r="A93" t="str">
+        <x:v>taronga-ferry-official</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>F2 Taronga Zoo Ferry</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D93" t="str">
+        <x:v>https://transportnsw.info/routes/details/sydney-ferries/f2/090f2</x:v>
+      </x:c>
+      <x:c r="E93" t="str"/>
+      <x:c r="F93" t="str"/>
+      <x:c r="G93" t="str">
+        <x:v>Transport for NSW</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
-      <x:c r="A94" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">felons-manly-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B94" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Felons Manly</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C94" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">restaurant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D94" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">https://www.google.com/maps/search/?api=1&amp;query=Felons+Manly</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G94" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Google Maps</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A94"/>
+      <x:c r="B94"/>
+      <x:c r="C94"/>
+      <x:c r="D94"/>
+      <x:c r="G94"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" t="inlineStr">
@@ -10884,7 +10727,7 @@
         <x:v>约 ¥4,375</x:v>
       </x:c>
       <x:c r="D6" s="2" t="str">
-        <x:v>Ledger snapshot 已确认活动约 ¥14,865.76：Reef Magic ¥5,260、Puffing Billy ¥2,352、Billy Tea A$956、观鲸 A$340.20、Opera House A$215；另留可选小门票预算</x:v>
+        <x:v>Ledger snapshot 已确认活动约 ¥14,865.76：Reef Magic ¥5,260、Puffing Billy ¥2,352、Billy Tea A$956、观鲸 A$340.20、Opera House A$215；另留 Taronga Zoo 和其他可选小门票预算</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -11200,7 +11043,7 @@
         <x:v>悉尼</x:v>
       </x:c>
       <x:c r="B10" s="28" t="str">
-        <x:v>Sydney Fish Market / Bondi / Manly</x:v>
+        <x:v>Sydney Fish Market / Bondi</x:v>
       </x:c>
       <x:c r="C10" s="28" t="str">
         <x:v>自由活动</x:v>
@@ -11213,6 +11056,26 @@
       </x:c>
       <x:c r="F10" s="28" t="str">
         <x:v>餐饮另计，不放入门票活动</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="40" customHeight="1">
+      <x:c r="A11" s="8" t="str">
+        <x:v>悉尼</x:v>
+      </x:c>
+      <x:c r="B11" s="8" t="str">
+        <x:v>Taronga Zoo Sydney</x:v>
+      </x:c>
+      <x:c r="C11" s="8" t="str">
+        <x:v>待订</x:v>
+      </x:c>
+      <x:c r="D11" s="8" t="str">
+        <x:v>官网成人线上价 A$51.30 × 4</x:v>
+      </x:c>
+      <x:c r="E11" s="8" t="str">
+        <x:v>约 ¥985</x:v>
+      </x:c>
+      <x:c r="F11" s="8" t="str">
+        <x:v>D15 使用；动物园门票与 F2 渡轮分开，线上价按官网当前信息记录</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -11541,10 +11404,8 @@
           <x:t xml:space="preserve">Darling Harbour / Pyrmont</x:t>
         </x:is>
       </x:c>
-      <x:c r="H7" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">适合 Darling Harbour、观鲸、Manly Ferry、CBD、QVB、Sydney Fish Market 和海港夜景；酒店官方地址为 Pyrmont Street / Darling Harbour</x:t>
-        </x:is>
+      <x:c r="H7" s="2" t="str">
+        <x:v>适合 Darling Harbour、观鲸、Taronga Zoo Ferry、CBD、QVB、Sydney Fish Market 和海港夜景；酒店官方地址为 Pyrmont Street / Darling Harbour</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -11719,38 +11580,38 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">灵活餐饮</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Prawn Star / Hello Auntie / Sydney Fish Market 等 food moments</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D7 / D10 / D12 / D14 / D15</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">餐饮点多数不提前锁死。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E5" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Prawn Star 可看是否需要订位；Hello Auntie 为 D12 晚餐备选；Sydney Fish Market 自由活动；Icebergs / Bondi Bistro 因 Totti’s 已订降级为备选；Hugos / Felons Manly 不建议锁死；Lune Croissanterie 看排队和路线。</x:t>
-        </x:is>
+      <x:c r="A5" s="2" t="str">
+        <x:v>建议提前购买</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="str">
+        <x:v>Taronga Zoo Sydney 门票</x:v>
+      </x:c>
+      <x:c r="C5" s="2" t="str">
+        <x:v>D15｜8/12</x:v>
+      </x:c>
+      <x:c r="D5" s="2" t="str">
+        <x:v>官网线上价低于现场价；确定行程后购买。</x:v>
+      </x:c>
+      <x:c r="E5" s="2" t="str">
+        <x:v>动物园冬季 09:30 开门；F2 渡轮与动物园门票分开，出发前查看当天班次。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="2" t="n"/>
-      <x:c r="B6" s="2" t="n"/>
-      <x:c r="C6" s="2" t="n"/>
-      <x:c r="D6" s="2" t="n"/>
-      <x:c r="E6" s="2" t="n"/>
+      <x:c r="A6" s="2" t="str">
+        <x:v>灵活餐饮</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="str">
+        <x:v>Prawn Star / Hello Auntie / Sydney Fish Market 等 food moments</x:v>
+      </x:c>
+      <x:c r="C6" s="2" t="str">
+        <x:v>D7 / D10 / D12 / D14</x:v>
+      </x:c>
+      <x:c r="D6" s="2" t="str">
+        <x:v>餐饮点多数不提前锁死。</x:v>
+      </x:c>
+      <x:c r="E6" s="2" t="str">
+        <x:v>Prawn Star 可看是否需要订位；Hello Auntie 为 D12 晚餐备选；Sydney Fish Market 自由活动；Icebergs / Bondi Bistro 因 Totti’s 已订降级为备选；Lune Croissanterie 看排队和路线。</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="2" t="n"/>
@@ -12208,31 +12069,21 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D15 Manly + 告别</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">café / Single O / Toby’s Estate</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Manly fish &amp; chips / Hugos / Felons Manly</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16:40 左右出发去 Circular Quay；17:00–17:20 外面拍日落光线；17:30 入座；注意带外套</x:t>
-        </x:is>
+    <x:row r="16" ht="40" customHeight="1">
+      <x:c r="A16" s="8" t="str">
+        <x:v>D15 Taronga Zoo + 告别</x:v>
+      </x:c>
+      <x:c r="B16" s="8" t="str">
+        <x:v>café / Single O / Toby’s Estate</x:v>
+      </x:c>
+      <x:c r="C16" s="8" t="str">
+        <x:v>Taronga Zoo Café / 自带轻食 / Circular Quay casual lunch</x:v>
+      </x:c>
+      <x:c r="D16" s="8" t="str">
+        <x:v>Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+      </x:c>
+      <x:c r="E16" s="8" t="str">
+        <x:v>上午搭 F2 Ferry 往返 Taronga Zoo；下午采购并整理 TRS；16:40 出发去 Circular Quay</x:v>
       </x:c>
     </x:row>
     <x:row r="17">

</xml_diff>

<commit_message>
feat: add QVM winter night market to D1
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R04738e3f54ee47d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R8ae9fe880a1444f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R163255b5ce384fda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R3366935c4240479b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R3398de61b0564ae9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R6933ad6862944364"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R867aec21b6f34b97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="Ra1f5b7fe54a844e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="Re095f495fa3d4d45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="R1e998734660347c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="Rf113a851b23144cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R136e9e968a864a6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R994df13ae0ef4ed8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R06ebb180737f4900"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="Rea22b1456add4751"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R437e6b07e4d0435e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R9743cc6874354fa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R653df487c08e4592"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -721,10 +721,8 @@
           <x:t xml:space="preserve">抵达墨尔本，CBD 轻量 city walk</x:t>
         </x:is>
       </x:c>
-      <x:c r="I3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">05:55 抵达，入境、休息；CBD city walk：Degraves Lane、Flinders Street、State Library、Hosier Lane、Southbank / Yarra River 夜景，按体力缩短。</x:t>
-        </x:is>
+      <x:c r="I3" t="str">
+        <x:v>05:55 抵达，入境、休息；白天按体力安排 Degraves Lane、Flinders Street、State Library、Hosier Lane，下午优先回酒店休息；17:30-19:30 QVM Winter Night Market（2026 冬季周三限定），结束后直接回酒店。</x:v>
       </x:c>
       <x:c r="J3" t="inlineStr">
         <x:is>
@@ -2348,35 +2346,23 @@
       <x:c r="B9" t="n">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="C9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">傍晚</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Southbank / Yarra River</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">河边散步</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">墨尔本夜景、城市氛围</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">轻松走 20-40 分钟即可；拍照：Yarra River 倒影、Flinders 夜灯</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">southbank-map,flinders-street-map</x:t>
-        </x:is>
+      <x:c r="C9" t="str">
+        <x:v>傍晚</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>Queen Victoria Market</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>17:30-19:30 QVM Winter Night Market</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>冬季周三限定夜市</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>官方场次 17:00-22:00，免费入场、免预约；落地日建议 17:30 前到，按体力逛 30-120 分钟，穿防风保暖外套。</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>qvm-map,qvm-winter-night-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2388,35 +2374,23 @@
       <x:c r="B10" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="C10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">晚上</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Southbank / CBD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">简单晚餐</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">落地日收尾</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">不订正式餐厅，早点回酒店休息；拍照：雨后街灯反光 / 河岸夜景</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">southbank-map,riverland-map</x:t>
-        </x:is>
+      <x:c r="C10" t="str">
+        <x:v>晚上</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>QVM → Oaks Melbourne on Market Hotel</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>夜市用餐后直接回酒店休息</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>落地日收尾</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>不再另订正式餐厅；如体力不足，可只逛 30-60 分钟后返回酒店。</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>qvm-map,oaks-market-map,qvm-winter-night-market-official</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2438,25 +2412,17 @@
           <x:t xml:space="preserve">饮食安排</x:t>
         </x:is>
       </x:c>
-      <x:c r="E11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">早餐：CBD café / Operator25（可选Brunch）；午餐：Degraves Lane / CBD 简餐 / Pho Tùng（可选）；晚餐：Southbank Riverland / Ponyfish Island / CBD 简餐</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">每日餐食参考</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">轻恢复</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">southbank-map,riverland-map,ponyfish-map,operator25-map,pho-tung-map,degraves-map</x:t>
-        </x:is>
+      <x:c r="E11" t="str">
+        <x:v>早餐：CBD café / Operator25（可选 Brunch）；午餐：Degraves Lane / CBD 简餐 / Pho Tùng（可选）；晚餐：QVM Winter Night Market 街头热食（主）/ CBD 简餐（体力不足）</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>每日餐食参考</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>夜市作为晚餐，优先选热食；不再另排 Southbank 正式晚餐。</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>qvm-map,qvm-winter-night-market-official,operator25-map,pho-tung-map,degraves-map</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -10593,6 +10559,25 @@
       <x:c r="F128" s="8"/>
       <x:c r="G128" s="8" t="str">
         <x:v>每日明确票券状态</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" t="str">
+        <x:v>qvm-winter-night-market-official</x:v>
+      </x:c>
+      <x:c r="B129" t="str">
+        <x:v>QVM Winter Night Market 2026</x:v>
+      </x:c>
+      <x:c r="C129" t="str">
+        <x:v>official</x:v>
+      </x:c>
+      <x:c r="D129" t="str">
+        <x:v>https://whatson.melbourne.vic.gov.au/things-to-do/winter-night-market</x:v>
+      </x:c>
+      <x:c r="E129"/>
+      <x:c r="F129"/>
+      <x:c r="G129" t="str">
+        <x:v>City of Melbourne：2026-07-29 17:00-22:00，免费，免预约；QVM 官网确认每周三 6/3-8/26。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11707,15 +11692,11 @@
           <x:t xml:space="preserve">Degraves Lane / CBD 简餐 / Pho Tùng（可选）</x:t>
         </x:is>
       </x:c>
-      <x:c r="D2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Southbank Riverland / Ponyfish Island / CBD 简餐</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">轻恢复</x:t>
-        </x:is>
+      <x:c r="D2" t="str">
+        <x:v>QVM Winter Night Market 街头热食 / CBD 简餐（体力不足）</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>落地日轻量安排；下午优先回酒店休息；17:30-19:30 逛夜市，按体力缩短。</x:v>
       </x:c>
     </x:row>
     <x:row r="3">

</xml_diff>

<commit_message>
content: shorten daily itinerary summaries
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -671,7 +671,7 @@
       </x:c>
       <x:c r="I2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">出发，香港转机 1h35m，夜航飞墨尔本</x:t>
+          <x:t xml:space="preserve">经香港转机，夜航前往墨尔本。</x:t>
         </x:is>
       </x:c>
       <x:c r="J2" t="inlineStr">
@@ -761,7 +761,7 @@
         <x:v>抵达墨尔本，CBD + Carlton + QVM 冬季夜市</x:v>
       </x:c>
       <x:c r="I3" t="str">
-        <x:v>05:55 抵达，入境、休息；白天按体力安排 Degraves Lane、Flinders Street、State Library、Carlton / Lygon Street（Little Italy）与 Hosier Lane；下午保留酒店休息；17:30-19:30 QVM Winter Night Market（2026 冬季周三限定），结束后直接回酒店。</x:v>
+        <x:v>落地恢复，轻走 CBD；晚间逛 QVM 冬季夜市。</x:v>
       </x:c>
       <x:c r="J3" t="inlineStr">
         <x:is>
@@ -850,7 +850,7 @@
         <x:v>Puffing Billy + Sassafras + Fitzroy</x:v>
       </x:c>
       <x:c r="I4" t="str">
-        <x:v>Klook / Oznara Puffing Billy + Sassafras 半日团已订；返回 343 Russell Street 后固定前往 Fitzroy，沿 Brunswick Street 与 Gertrude Street 漫步，晚上整理大洋路行李。</x:v>
+        <x:v>蒸汽小火车半日，下午漫步 Fitzroy。</x:v>
       </x:c>
       <x:c r="J4" t="inlineStr">
         <x:is>
@@ -942,7 +942,7 @@
       </x:c>
       <x:c r="I5" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">退房后前往墨尔本机场取车，大件行李寄存，只带登机箱上大洋路；Torquay、Bells Beach、Split Point Lighthouse、Lorne、Kennett River、Apollo Bay</x:t>
+          <x:t xml:space="preserve">机场取车轻装上路，沿海开到 Apollo Bay。</x:t>
         </x:is>
       </x:c>
       <x:c r="J5" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </x:c>
       <x:c r="I6" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Maits Rest Rainforest + Gibson Steps + Twelve Apostles + Loch Ard Gorge + Port Campbell；晚餐买食材，抵达后按时间和天气决定户外 public electric BBQ 或 villa 厨房自炊</x:t>
+          <x:t xml:space="preserve">穿过雨林走向十二使徒岩，傍晚抵达 Port Campbell。</x:t>
         </x:is>
       </x:c>
       <x:c r="J6" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </x:c>
       <x:c r="I7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Twelve Apostles / Loch Ard Gorge 清晨补拍 + London Arch + The Grotto + Colac 中转 + 机场还车 + 取回寄存大件行李 + 入住机场酒店</x:t>
+          <x:t xml:space="preserve">清晨补拍海岸，走内陆线返回墨尔本机场。</x:t>
         </x:is>
       </x:c>
       <x:c r="J7" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </x:c>
       <x:c r="I8" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">VA1291 飞凯恩斯 + Esplanade Lagoon + 夜市</x:t>
+          <x:t xml:space="preserve">从冬季飞进热带，傍晚漫步凯恩斯海滨。</x:t>
         </x:is>
       </x:c>
       <x:c r="J8" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </x:c>
       <x:c r="I9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Reef Magic 外礁平台一日游已订 ¥5,260：Outer Reef Pontoon，浮潜 / 半潜艇 / 玻璃底船 / 平台体验</x:t>
+          <x:t xml:space="preserve">全天留给大堡礁外礁平台与海上体验。</x:t>
         </x:is>
       </x:c>
       <x:c r="J9" t="inlineStr">
@@ -1407,7 +1407,7 @@
       </x:c>
       <x:c r="I10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Billy Tea Daintree：Daintree River（鳄鱼）+ Rainforest + Cape Tribulation（雨林入海）+ Daintree Ice Cream</x:t>
+          <x:t xml:space="preserve">沿丹翠河深入雨林，在 Cape Tribulation 看雨林入海。</x:t>
         </x:is>
       </x:c>
       <x:c r="J10" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </x:c>
       <x:c r="I11" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lake Eacham（火山湖）+ Curtain Fig Tree（巨树）+ Yungaburra + Millaa Millaa Falls（主瀑布）</x:t>
+          <x:t xml:space="preserve">轻量自驾串联火山湖、巨树、高原小镇与瀑布。</x:t>
         </x:is>
       </x:c>
       <x:c r="J11" t="inlineStr">
@@ -1590,7 +1590,7 @@
         <x:v>Rusty’s Market + Palm Cove + 休息整理</x:v>
       </x:c>
       <x:c r="I12" t="str">
-        <x:v>Rusty’s Market + 休息、洗衣与行李整理 + Palm Cove 海滨与棕榈大道 + 返回凯恩斯早晚餐。</x:v>
+        <x:v>逛 Rusty’s Market，休整后去 Palm Cove 看海。</x:v>
       </x:c>
       <x:c r="J12" t="inlineStr">
         <x:is>
@@ -1679,7 +1679,7 @@
         <x:v>转场悉尼，Barangaroo + The Rocks + 海港夜景</x:v>
       </x:c>
       <x:c r="I13" t="str">
-        <x:v>JQ953 飞悉尼；酒店休息后沿 Barangaroo Reserve / Wulugul Walk 前往 The Rocks，最后到 Circular Quay 看夜景。</x:v>
+        <x:v>飞抵悉尼休息后，经 Barangaroo 走向海港夜景。</x:v>
       </x:c>
       <x:c r="J13" t="inlineStr">
         <x:is>
@@ -1771,7 +1771,7 @@
       </x:c>
       <x:c r="I14" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Circular Quay + Sydney Opera House 中文导览 9:30 已订 + Man O’War Steps + Royal Botanic Garden + Mrs Macquarie’s Chair + QVB</x:t>
+          <x:t xml:space="preserve">从歌剧院导览一路步行到花园、经典机位与 QVB。</x:t>
         </x:is>
       </x:c>
       <x:c r="J14" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </x:c>
       <x:c r="I15" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Grand Pacific Drive + Bald Hill + Sea Cliff Bridge + Kiama + Gerringong；时间、天气和体力允许时再延伸 Kangaroo Valley。</x:t>
+          <x:t xml:space="preserve">沿 Grand Pacific Drive 南下，串联海崖桥与南海岸小镇。</x:t>
         </x:is>
       </x:c>
       <x:c r="J15" t="inlineStr">
@@ -1957,7 +1957,7 @@
       </x:c>
       <x:c r="I16" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Sydney Harbour 公共 F2 Ferry + Taronga Zoo + Bondi Beach / Icebergs / Tamarama；Totti’s Bondi 18:30 晚餐已订</x:t>
+          <x:t xml:space="preserve">上午看澳洲动物，下午走 Bondi 海岸，晚上吃 Totti’s。</x:t>
         </x:is>
       </x:c>
       <x:c r="J16" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </x:c>
       <x:c r="I17" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">早上看状态决定是否搭 F1 Ferry 去 Manly；随后 QVB / Chemist Warehouse 最后采购、TRS / 行李整理；Cafe Sydney 17:30 Outdoor Terrace Dining 告别晚餐已订</x:t>
+          <x:t xml:space="preserve">早上按状态决定 Manly，下午采购整理，傍晚 Cafe Sydney。</x:t>
         </x:is>
       </x:c>
       <x:c r="J17" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </x:c>
       <x:c r="I18" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">返程 + TRS退税</x:t>
+          <x:t xml:space="preserve">完成 TRS 与机场手续，启程回家。</x:t>
         </x:is>
       </x:c>
       <x:c r="J18" t="inlineStr">

</xml_diff>

<commit_message>
refactor: polish itinerary copy for travellers
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="Raa7dfcbcfc314f2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="Ra3b4d579a1f3462c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R063960871c9644c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="Reb562c62a5a34f7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R4b10e12eca264ed2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R9ff73656fce54f7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R1af32aa126544d0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R65160bded75b4d45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R95b3d9f28dcd4b1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="Rcaf0662ad52f4884"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="Rec59b5d3e81645a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R41015571a2c145ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R24905560db084c24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="Ra588fa49be624df3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R4e37d463674e4a69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="Rd9fce5cbf2794b07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R7115d181bbcc4db3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R1c7f67636cd04c77"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -633,30 +633,20 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-28</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周二</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">上海 → 香港 → 墨尔本</x:t>
-        </x:is>
+      <x:c r="A2" t="str">
+        <x:v>d0</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>D0</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>2026-07-28</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>上海 → 香港 → 墨尔本</x:v>
       </x:c>
       <x:c r="F2" t="n">
         <x:v>31.2304</x:v>
@@ -664,92 +654,58 @@
       <x:c r="G2" t="n">
         <x:v>121.4737</x:v>
       </x:c>
-      <x:c r="H2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">上海出发，香港转机飞墨尔本</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">经香港转机，夜航前往墨尔本。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">飞机上</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">夜航为主，机场和机舱温差明显。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">随身带薄外套、颈枕、充电线和第一天入境资料。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/d0-shanghai-departure.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">上海机场夜间出发</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">航班 / 机场转场</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">按国际航班时间倒推，提前 3 小时到机场</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">flight-cathay</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">shanghai-pudong-airport-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">flight-cathay</x:t>
-        </x:is>
+      <x:c r="H2" t="str">
+        <x:v>启程澳洲：香港转机，夜航墨尔本</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>经香港转机，夜航前往墨尔本。</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
+        <x:v>飞机上</x:v>
+      </x:c>
+      <x:c r="K2" t="str">
+        <x:v>夜航为主，机场和机舱温差明显。</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>随身带薄外套、颈枕和充电线；入境与酒店资料放在随身包。</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
+        <x:v>/itinerary/d0-shanghai-departure.png</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>上海机场夜间出发</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
+        <x:v>航班 / 机场转场</x:v>
+      </x:c>
+      <x:c r="P2" t="str">
+        <x:v>按国际航班时间倒推，提前 3 小时到机场</x:v>
+      </x:c>
+      <x:c r="Q2" t="str">
+        <x:v>flight-cathay</x:v>
+      </x:c>
+      <x:c r="R2" t="str">
+        <x:v>shanghai-pudong-airport-map</x:v>
+      </x:c>
+      <x:c r="S2" t="str">
+        <x:v>flight-cathay</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-29</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周三</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">墨尔本</x:t>
-        </x:is>
+      <x:c r="A3" t="str">
+        <x:v>d1</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>D1</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>墨尔本</x:v>
       </x:c>
       <x:c r="F3" t="n">
         <x:v>-37.8136</x:v>
@@ -758,87 +714,57 @@
         <x:v>144.9631</x:v>
       </x:c>
       <x:c r="H3" t="str">
-        <x:v>抵达墨尔本，CBD + Carlton + QVM 冬季夜市</x:v>
+        <x:v>初到墨尔本：CBD、Carlton 与 QVM 冬季夜市</x:v>
       </x:c>
       <x:c r="I3" t="str">
-        <x:v>落地恢复，轻走 CBD；晚间逛 QVM 冬季夜市。</x:v>
-      </x:c>
-      <x:c r="J3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Oaks Melbourne on Market Hotel</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">墨尔本冬季约 6-14°C，早晚冷，多风，偶有阵雨。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">羽绒服或防风外套、毛衣、长裤、防水鞋。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/melbourne-city-morning.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">墨尔本清晨城市街景</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">机场接送 + 步行 / 市内交通</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">05:55 抵达；入境后直接前往 CBD</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">oaks-market-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">mel-airport-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">no-fixed-ticket</x:t>
-        </x:is>
+        <x:v>抵达后慢慢恢复，逛过 CBD 与 Carlton，晚上去 QVM 冬季夜市吃晚餐。</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>Oaks Melbourne on Market Hotel</x:v>
+      </x:c>
+      <x:c r="K3" t="str">
+        <x:v>墨尔本冬季约 6-14°C，早晚冷，多风，偶有阵雨。</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>羽绒服或防风外套、毛衣、长裤、防水鞋。</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>/itinerary/melbourne-city-morning.png</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>墨尔本清晨城市街景</x:v>
+      </x:c>
+      <x:c r="O3" t="str">
+        <x:v>机场接送 + 步行 / 市内交通</x:v>
+      </x:c>
+      <x:c r="P3" t="str">
+        <x:v>05:55 抵达；入境后直接前往 CBD</x:v>
+      </x:c>
+      <x:c r="Q3" t="str">
+        <x:v>oaks-market-map</x:v>
+      </x:c>
+      <x:c r="R3" t="str">
+        <x:v>mel-airport-map</x:v>
+      </x:c>
+      <x:c r="S3" t="str">
+        <x:v>no-fixed-ticket</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-30</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周四</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">墨尔本 + Belgrave</x:t>
-        </x:is>
+      <x:c r="A4" t="str">
+        <x:v>d2</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>D2</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>墨尔本 + Belgrave</x:v>
       </x:c>
       <x:c r="F4" t="n">
         <x:v>-37.8136</x:v>
@@ -847,87 +773,57 @@
         <x:v>144.9631</x:v>
       </x:c>
       <x:c r="H4" t="str">
-        <x:v>Puffing Billy + Sassafras + Fitzroy</x:v>
+        <x:v>墨尔本近郊：Puffing Billy、Sassafras 与 Fitzroy</x:v>
       </x:c>
       <x:c r="I4" t="str">
-        <x:v>蒸汽小火车半日，下午漫步 Fitzroy。</x:v>
-      </x:c>
-      <x:c r="J4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Oaks Melbourne on Market Hotel</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">墨尔本冬季约 6-14°C，早晚冷，多风，偶有阵雨。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">防风外套比单纯厚毛衣更实用，雨天鞋子尽量防水。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/d2-puffing-billy-railway.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Puffing Billy 蒸汽小火车穿过 Dandenong Ranges 森林</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">半日团接驳车 + Puffing Billy 蒸汽火车</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">按通知的集合时间，提前 15 分钟到 343 Russell Street</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">oaks-market-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">russell-343-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">puffing-billy-official</x:t>
-        </x:is>
+        <x:v>上午乘 Puffing Billy 穿行山林，下午在 Fitzroy 看街区与小店。</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>Oaks Melbourne on Market Hotel</x:v>
+      </x:c>
+      <x:c r="K4" t="str">
+        <x:v>墨尔本冬季约 6-14°C，早晚冷，多风，偶有阵雨。</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>防风外套比单纯厚毛衣更实用，雨天鞋子尽量防水。</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>/itinerary/d2-puffing-billy-railway.png</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>Puffing Billy 蒸汽小火车穿过 Dandenong Ranges 森林</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
+        <x:v>半日团接驳车 + Puffing Billy 蒸汽火车</x:v>
+      </x:c>
+      <x:c r="P4" t="str">
+        <x:v>按通知的集合时间，提前 15 分钟到 343 Russell Street</x:v>
+      </x:c>
+      <x:c r="Q4" t="str">
+        <x:v>oaks-market-map</x:v>
+      </x:c>
+      <x:c r="R4" t="str">
+        <x:v>russell-343-map</x:v>
+      </x:c>
+      <x:c r="S4" t="str">
+        <x:v>puffing-billy-official</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-07-31</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周五</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">墨尔本机场 → Apollo Bay</x:t>
-        </x:is>
+      <x:c r="A5" t="str">
+        <x:v>d3</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>D3</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>2026-07-31</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>墨尔本机场 → Apollo Bay</x:v>
       </x:c>
       <x:c r="F5" t="n">
         <x:v>-38.7599</x:v>
@@ -935,92 +831,58 @@
       <x:c r="G5" t="n">
         <x:v>143.6692</x:v>
       </x:c>
-      <x:c r="H5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">大洋路 Road Trip Day 1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">机场取车轻装上路，沿海开到 Apollo Bay。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Seaview Motel &amp; Apartments</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">维州南海岸冬季多风，体感比温度更冷。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">防风外套、长裤、防滑鞋；车上备水和零食。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/d3-great-ocean-road-lorne.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">大洋路早段海岸公路与灯塔</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">自驾 · 墨尔本机场取车</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">08:00 前退房出发，预留机场取车时间</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">seaview-motel-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">mel-airport-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">no-fixed-ticket</x:t>
-        </x:is>
+      <x:c r="H5" t="str">
+        <x:v>驶上大洋路：Torquay、Lorne 到 Apollo Bay</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>机场取车后沿海向西，途经 Torquay、Lorne，傍晚住进 Apollo Bay。</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>Seaview Motel &amp; Apartments</x:v>
+      </x:c>
+      <x:c r="K5" t="str">
+        <x:v>维州南海岸冬季多风，体感比温度更冷。</x:v>
+      </x:c>
+      <x:c r="L5" t="str">
+        <x:v>防风外套、长裤、防滑鞋；车上备水和零食。</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
+        <x:v>/itinerary/d3-great-ocean-road-lorne.png</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>大洋路早段海岸公路与灯塔</x:v>
+      </x:c>
+      <x:c r="O5" t="str">
+        <x:v>自驾 · 墨尔本机场取车</x:v>
+      </x:c>
+      <x:c r="P5" t="str">
+        <x:v>08:00 前退房出发，预留机场取车时间</x:v>
+      </x:c>
+      <x:c r="Q5" t="str">
+        <x:v>seaview-motel-map</x:v>
+      </x:c>
+      <x:c r="R5" t="str">
+        <x:v>mel-airport-map</x:v>
+      </x:c>
+      <x:c r="S5" t="str">
+        <x:v>no-fixed-ticket</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d4</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D4</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-01</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周六</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Apollo Bay → Port Campbell</x:t>
-        </x:is>
+      <x:c r="A6" t="str">
+        <x:v>d4</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>D4</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>2026-08-01</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>周六</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>Apollo Bay → Port Campbell</x:v>
       </x:c>
       <x:c r="F6" t="n">
         <x:v>-38.6191</x:v>
@@ -1028,92 +890,58 @@
       <x:c r="G6" t="n">
         <x:v>142.9956</x:v>
       </x:c>
-      <x:c r="H6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">十二使徒岩与 Loch Ard Gorge</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">穿过雨林走向十二使徒岩，傍晚抵达 Port Campbell。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Southern Ocean Villas</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">海岸风大，步道和台阶雨后湿滑。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">防风外套、防水鞋；拍照时不要太靠近海浪。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/d4-twelve-apostles-gorge.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">十二使徒岩与峡谷海岸</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">自驾 · 大洋路海岸段</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">08:30 前离开 Apollo Bay</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">southern-ocean-villas-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">maits-rest-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">no-fixed-ticket</x:t>
-        </x:is>
+      <x:c r="H6" t="str">
+        <x:v>大洋路海岸：雨林、十二使徒岩与 Loch Ard Gorge</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>从雨林步道驶向十二使徒岩，在 Loch Ard Gorge 慢慢看海岸地貌。</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>Southern Ocean Villas</x:v>
+      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>海岸风大，步道和台阶雨后湿滑。</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>防风外套、防水鞋；拍照时不要太靠近海浪。</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
+        <x:v>/itinerary/d4-twelve-apostles-gorge.png</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>十二使徒岩与峡谷海岸</x:v>
+      </x:c>
+      <x:c r="O6" t="str">
+        <x:v>自驾 · 大洋路海岸段</x:v>
+      </x:c>
+      <x:c r="P6" t="str">
+        <x:v>08:30 前离开 Apollo Bay</x:v>
+      </x:c>
+      <x:c r="Q6" t="str">
+        <x:v>southern-ocean-villas-map</x:v>
+      </x:c>
+      <x:c r="R6" t="str">
+        <x:v>maits-rest-map</x:v>
+      </x:c>
+      <x:c r="S6" t="str">
+        <x:v>no-fixed-ticket</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d5</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D5</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-02</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周日</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Port Campbell → 墨尔本机场</x:t>
-        </x:is>
+      <x:c r="A7" t="str">
+        <x:v>d5</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>D5</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>周日</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>Port Campbell → 墨尔本机场</x:v>
       </x:c>
       <x:c r="F7" t="n">
         <x:v>-37.669</x:v>
@@ -1121,92 +949,58 @@
       <x:c r="G7" t="n">
         <x:v>144.841</x:v>
       </x:c>
-      <x:c r="H7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">清晨补拍，内陆回机场</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">清晨补拍海岸，走内陆线返回墨尔本机场。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Holiday Inn Melbourne Airport</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">早晨海边冷，回程时间长。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">早上防风保暖，下午回机场前预留加油和还车时间。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/d5-port-campbell-morning.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Port Campbell 清晨海岸</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">自驾 · 内陆回墨尔本机场</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">08:00 前离开 Port Campbell，17:00 前还车更稳</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">holiday-inn-airport-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">twelve-apostles-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">no-fixed-ticket</x:t>
-        </x:is>
+      <x:c r="H7" t="str">
+        <x:v>告别大洋路：清晨海岸与内陆返程</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>清晨再看一眼海岸，经 Colac 走内陆线返回墨尔本机场。</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:v>Holiday Inn Melbourne Airport</x:v>
+      </x:c>
+      <x:c r="K7" t="str">
+        <x:v>早晨海边冷，回程时间长。</x:v>
+      </x:c>
+      <x:c r="L7" t="str">
+        <x:v>早上防风保暖，下午回机场前预留加油和还车时间。</x:v>
+      </x:c>
+      <x:c r="M7" t="str">
+        <x:v>/itinerary/d5-port-campbell-morning.png</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>Port Campbell 清晨海岸</x:v>
+      </x:c>
+      <x:c r="O7" t="str">
+        <x:v>自驾 · 内陆回墨尔本机场</x:v>
+      </x:c>
+      <x:c r="P7" t="str">
+        <x:v>08:00 前离开 Port Campbell，17:00 前还车更稳</x:v>
+      </x:c>
+      <x:c r="Q7" t="str">
+        <x:v>holiday-inn-airport-map</x:v>
+      </x:c>
+      <x:c r="R7" t="str">
+        <x:v>twelve-apostles-map</x:v>
+      </x:c>
+      <x:c r="S7" t="str">
+        <x:v>no-fixed-ticket</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d6</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D6</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-03</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周一</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">墨尔本 → 凯恩斯</x:t>
-        </x:is>
+      <x:c r="A8" t="str">
+        <x:v>d6</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>D6</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>2026-08-03</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>墨尔本 → 凯恩斯</x:v>
       </x:c>
       <x:c r="F8" t="n">
         <x:v>-16.9186</x:v>
@@ -1214,92 +1008,58 @@
       <x:c r="G8" t="n">
         <x:v>145.7781</x:v>
       </x:c>
-      <x:c r="H8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">飞进热带，Esplanade Lagoon</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">从冬季飞进热带，傍晚漫步凯恩斯海滨。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Southern Cross Atrium Apartments</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">凯恩斯约 17-26°C，旱季，阳光充足。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">短袖、防晒衣、墨镜、帽子；机舱和室内空调可能冷。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/cairns-reef-lagoon.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">凯恩斯热带海岸</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">航班 / 机场转场</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">04:00 前从机场酒店步行或接驳至航站楼</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">southern-cross-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">mel-airport-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">virgin-australia-official</x:t>
-        </x:is>
+      <x:c r="H8" t="str">
+        <x:v>抵达凯恩斯：Esplanade Lagoon 与热带夜市</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>从墨尔本飞到凯恩斯，下午在 Esplanade Lagoon 放松，晚上逛夜市。</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>Southern Cross Atrium Apartments</x:v>
+      </x:c>
+      <x:c r="K8" t="str">
+        <x:v>凯恩斯约 17-26°C，旱季，阳光充足。</x:v>
+      </x:c>
+      <x:c r="L8" t="str">
+        <x:v>短袖、防晒衣、墨镜、帽子；机舱和室内空调可能冷。</x:v>
+      </x:c>
+      <x:c r="M8" t="str">
+        <x:v>/itinerary/cairns-reef-lagoon.png</x:v>
+      </x:c>
+      <x:c r="N8" t="str">
+        <x:v>凯恩斯热带海岸</x:v>
+      </x:c>
+      <x:c r="O8" t="str">
+        <x:v>航班 / 机场转场</x:v>
+      </x:c>
+      <x:c r="P8" t="str">
+        <x:v>04:00 前从机场酒店步行或接驳至航站楼</x:v>
+      </x:c>
+      <x:c r="Q8" t="str">
+        <x:v>southern-cross-map</x:v>
+      </x:c>
+      <x:c r="R8" t="str">
+        <x:v>mel-airport-map</x:v>
+      </x:c>
+      <x:c r="S8" t="str">
+        <x:v>virgin-australia-official</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d7</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D7</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-04</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周二</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">凯恩斯</x:t>
-        </x:is>
+      <x:c r="A9" t="str">
+        <x:v>d7</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>D7</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>2026-08-04</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>凯恩斯</x:v>
       </x:c>
       <x:c r="F9" t="n">
         <x:v>-16.9186</x:v>
@@ -1307,92 +1067,58 @@
       <x:c r="G9" t="n">
         <x:v>145.7781</x:v>
       </x:c>
-      <x:c r="H9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Reef Magic 外礁一日游</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">全天留给大堡礁外礁平台与海上体验。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Southern Cross Atrium Apartments</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">海上日晒强，船舱空调可能很冷。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">防晒衣比防晒霜更重要，带薄外套并提前吃晕船药。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/d7-great-barrier-reef-pontoon.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">大堡礁外礁平台</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">步行 / 打车至码头 + Reef Magic 游船</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">按船票集合时间，提前 45 分钟到 Reef Fleet Terminal</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">southern-cross-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">reef-fleet-terminal-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">reef-magic-official</x:t>
-        </x:is>
+      <x:c r="H9" t="str">
+        <x:v>奔赴外礁：Reef Magic 大堡礁一日</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>在 Reef Magic 外礁平台体验浮潜、半潜艇与大堡礁海上风景。</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>Southern Cross Atrium Apartments</x:v>
+      </x:c>
+      <x:c r="K9" t="str">
+        <x:v>海上日晒强，船舱空调可能很冷。</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>防晒衣比防晒霜更重要，带薄外套并提前吃晕船药。</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
+        <x:v>/itinerary/d7-great-barrier-reef-pontoon.png</x:v>
+      </x:c>
+      <x:c r="N9" t="str">
+        <x:v>大堡礁外礁平台</x:v>
+      </x:c>
+      <x:c r="O9" t="str">
+        <x:v>步行 / 打车至码头 + Reef Magic 游船</x:v>
+      </x:c>
+      <x:c r="P9" t="str">
+        <x:v>按船票集合时间，提前 45 分钟到 Reef Fleet Terminal</x:v>
+      </x:c>
+      <x:c r="Q9" t="str">
+        <x:v>southern-cross-map</x:v>
+      </x:c>
+      <x:c r="R9" t="str">
+        <x:v>reef-fleet-terminal-map</x:v>
+      </x:c>
+      <x:c r="S9" t="str">
+        <x:v>reef-magic-official</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d8</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D8</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-05</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周三</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">丹翠雨林</x:t>
-        </x:is>
+      <x:c r="A10" t="str">
+        <x:v>d8</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>D8</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>2026-08-05</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>丹翠雨林</x:v>
       </x:c>
       <x:c r="F10" t="n">
         <x:v>-16.1705</x:v>
@@ -1400,92 +1126,58 @@
       <x:c r="G10" t="n">
         <x:v>145.4185</x:v>
       </x:c>
-      <x:c r="H10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">丹翠雨林 + Cape Tribulation 小团</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">沿丹翠河深入雨林，在 Cape Tribulation 看雨林入海。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Southern Cross Atrium Apartments</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">热带雨林湿润，车内空调可能冷。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">短袖、防晒、防蚊、帽子、薄外套；不建议下海游泳。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/daintree-rainforest.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">丹翠雨林</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Billy Tea 小团接驳车</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">06:40 前到酒店门口，06:55 集合</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">southern-cross-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">southern-cross-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">billy-tea-official</x:t>
-        </x:is>
+      <x:c r="H10" t="str">
+        <x:v>深入丹翠：雨林、河流与 Cape Tribulation</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>沿丹翠河进入雨林，在 Cape Tribulation 看雨林与海相接。</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>Southern Cross Atrium Apartments</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>热带雨林湿润，车内空调可能冷。</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>短袖、防晒、防蚊、帽子、薄外套；不建议下海游泳。</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>/itinerary/daintree-rainforest.png</x:v>
+      </x:c>
+      <x:c r="N10" t="str">
+        <x:v>丹翠雨林</x:v>
+      </x:c>
+      <x:c r="O10" t="str">
+        <x:v>Billy Tea 小团接驳车</x:v>
+      </x:c>
+      <x:c r="P10" t="str">
+        <x:v>06:40 前到酒店门口，06:55 集合</x:v>
+      </x:c>
+      <x:c r="Q10" t="str">
+        <x:v>southern-cross-map</x:v>
+      </x:c>
+      <x:c r="R10" t="str">
+        <x:v>southern-cross-map</x:v>
+      </x:c>
+      <x:c r="S10" t="str">
+        <x:v>billy-tea-official</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d9</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D9</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-06</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周四</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">阿瑟顿高原</x:t>
-        </x:is>
+      <x:c r="A11" t="str">
+        <x:v>d9</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>D9</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>2026-08-06</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>阿瑟顿高原</x:v>
       </x:c>
       <x:c r="F11" t="n">
         <x:v>-17.2706</x:v>
@@ -1493,92 +1185,58 @@
       <x:c r="G11" t="n">
         <x:v>145.5831</x:v>
       </x:c>
-      <x:c r="H11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">火山湖、巨树、小镇与瀑布</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">轻量自驾串联火山湖、巨树、高原小镇与瀑布。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Southern Cross Atrium Apartments</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">高原比凯恩斯海边更清凉。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">短袖加薄外套，瀑布和雨林步道注意防滑。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/d9-atherton-tablelands-waterfall.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">阿瑟顿高原瀑布</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">自驾 · 阿瑟顿高原</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">08:30 前取车出发</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">southern-cross-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">lake-eacham-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">no-fixed-ticket</x:t>
-        </x:is>
+      <x:c r="H11" t="str">
+        <x:v>阿瑟顿高原：火山湖、巨树与瀑布</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>自驾串联 Lake Eacham、Curtain Fig Tree、高原小镇与瀑布。</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>Southern Cross Atrium Apartments</x:v>
+      </x:c>
+      <x:c r="K11" t="str">
+        <x:v>高原比凯恩斯海边更清凉。</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>短袖加薄外套，瀑布和雨林步道注意防滑。</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>/itinerary/d9-atherton-tablelands-waterfall.png</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>阿瑟顿高原瀑布</x:v>
+      </x:c>
+      <x:c r="O11" t="str">
+        <x:v>自驾 · 阿瑟顿高原</x:v>
+      </x:c>
+      <x:c r="P11" t="str">
+        <x:v>08:30 前取车出发</x:v>
+      </x:c>
+      <x:c r="Q11" t="str">
+        <x:v>southern-cross-map</x:v>
+      </x:c>
+      <x:c r="R11" t="str">
+        <x:v>lake-eacham-map</x:v>
+      </x:c>
+      <x:c r="S11" t="str">
+        <x:v>no-fixed-ticket</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d10</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D10</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-07</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周五</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">凯恩斯休息日</x:t>
-        </x:is>
+      <x:c r="A12" t="str">
+        <x:v>d10</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>D10</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>2026-08-07</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>周五</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>凯恩斯休息日</x:v>
       </x:c>
       <x:c r="F12" t="n">
         <x:v>-16.9186</x:v>
@@ -1587,87 +1245,57 @@
         <x:v>145.7781</x:v>
       </x:c>
       <x:c r="H12" t="str">
-        <x:v>Rusty’s Market + Palm Cove + 休息整理</x:v>
+        <x:v>慢享凯恩斯：Rusty’s Market 与 Palm Cove</x:v>
       </x:c>
       <x:c r="I12" t="str">
-        <x:v>逛 Rusty’s Market，休整后去 Palm Cove 看海。</x:v>
-      </x:c>
-      <x:c r="J12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Southern Cross Atrium Apartments</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">凯恩斯约 17-26°C，户外热，室内空调冷。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">轻便夏装，随身带薄外套；今天不要再临时加长线。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/d10-cairns-rustys-market.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">凯恩斯市场与海滨</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">步行 / 市内短途交通</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09:00 前出门逛 Rusty's Market</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">southern-cross-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">rustys-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">no-fixed-ticket</x:t>
-        </x:is>
+        <x:v>上午逛 Rusty’s Market，午后休整，傍晚去 Palm Cove 看海。</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>Southern Cross Atrium Apartments</x:v>
+      </x:c>
+      <x:c r="K12" t="str">
+        <x:v>凯恩斯约 17-26°C，户外热，室内空调冷。</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>轻便夏装，随身带薄外套；傍晚海边有风。</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>/itinerary/d10-cairns-rustys-market.png</x:v>
+      </x:c>
+      <x:c r="N12" t="str">
+        <x:v>凯恩斯市场与海滨</x:v>
+      </x:c>
+      <x:c r="O12" t="str">
+        <x:v>步行 / 市内短途交通</x:v>
+      </x:c>
+      <x:c r="P12" t="str">
+        <x:v>09:00 前出门逛 Rusty's Market</x:v>
+      </x:c>
+      <x:c r="Q12" t="str">
+        <x:v>southern-cross-map</x:v>
+      </x:c>
+      <x:c r="R12" t="str">
+        <x:v>rustys-map</x:v>
+      </x:c>
+      <x:c r="S12" t="str">
+        <x:v>no-fixed-ticket</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d11</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D11</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-08</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周六</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">凯恩斯 → 悉尼</x:t>
-        </x:is>
+      <x:c r="A13" t="str">
+        <x:v>d11</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>D11</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>2026-08-08</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>周六</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>凯恩斯 → 悉尼</x:v>
       </x:c>
       <x:c r="F13" t="n">
         <x:v>-33.8688</x:v>
@@ -1676,87 +1304,57 @@
         <x:v>151.2093</x:v>
       </x:c>
       <x:c r="H13" t="str">
-        <x:v>转场悉尼，Barangaroo + The Rocks + 海港夜景</x:v>
+        <x:v>初到悉尼：Barangaroo、The Rocks 与海港夜景</x:v>
       </x:c>
       <x:c r="I13" t="str">
-        <x:v>飞抵悉尼休息后，经 Barangaroo 走向海港夜景。</x:v>
-      </x:c>
-      <x:c r="J13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Oaks Sydney Goldsbrough Suites</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悉尼约 9-18°C，早晚凉，海边防风。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">薄羽绒、风衣或卫衣；从凯恩斯上飞机随身带外套。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/d11-sydney-arrival-rocks.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悉尼 The Rocks 夜景</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">航班 / 机场转场 + 步行</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">按 JQ953 起飞时间，提前 2 小时到凯恩斯机场 T2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">oaks-sydney-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">cairns-airport-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">jetstar-official</x:t>
-        </x:is>
+        <x:v>飞抵悉尼后休息片刻，沿 Barangaroo、The Rocks 走到 Circular Quay 夜景。</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>Oaks Sydney Goldsbrough Suites</x:v>
+      </x:c>
+      <x:c r="K13" t="str">
+        <x:v>悉尼约 9-18°C，早晚凉，海边防风。</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>薄羽绒、风衣或卫衣；从凯恩斯上飞机随身带外套。</x:v>
+      </x:c>
+      <x:c r="M13" t="str">
+        <x:v>/itinerary/d11-sydney-arrival-rocks.png</x:v>
+      </x:c>
+      <x:c r="N13" t="str">
+        <x:v>悉尼 The Rocks 夜景</x:v>
+      </x:c>
+      <x:c r="O13" t="str">
+        <x:v>航班 / 机场转场 + 步行</x:v>
+      </x:c>
+      <x:c r="P13" t="str">
+        <x:v>按 JQ953 起飞时间，提前 2 小时到凯恩斯机场 T2</x:v>
+      </x:c>
+      <x:c r="Q13" t="str">
+        <x:v>oaks-sydney-map</x:v>
+      </x:c>
+      <x:c r="R13" t="str">
+        <x:v>cairns-airport-map</x:v>
+      </x:c>
+      <x:c r="S13" t="str">
+        <x:v>jetstar-official</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d12</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D12</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-09</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周日</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悉尼市区</x:t>
-        </x:is>
+      <x:c r="A14" t="str">
+        <x:v>d12</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>D12</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>2026-08-09</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>周日</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>悉尼市区</x:v>
       </x:c>
       <x:c r="F14" t="n">
         <x:v>-33.8688</x:v>
@@ -1765,87 +1363,57 @@
         <x:v>151.2093</x:v>
       </x:c>
       <x:c r="H14" t="str">
-        <x:v>歌剧院中文导览 + The Rocks Weekend Market</x:v>
+        <x:v>悉尼经典一日：歌剧院、The Rocks Weekend Market、植物园与 QVB</x:v>
       </x:c>
       <x:c r="I14" t="str">
-        <x:v>中文导览结束后步行逛 The Rocks 周末市集，再前往植物园、经典机位与 QVB。</x:v>
-      </x:c>
-      <x:c r="J14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Oaks Sydney Goldsbrough Suites</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悉尼冬季晴天概率较好，早晚凉。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">薄羽绒或风衣，海港边风大时注意保暖。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/d12-sydney-opera-garden.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悉尼歌剧院与植物园</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">步行 + 市内交通</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">08:45 前出门，09:15 前到 Sydney Opera House</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">oaks-sydney-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">opera-house-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">opera-house-official</x:t>
-        </x:is>
+        <x:v>从歌剧院中文导览出发，逛 The Rocks 周末市集，再沿植物园走到经典海港机位与 QVB。</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>Oaks Sydney Goldsbrough Suites</x:v>
+      </x:c>
+      <x:c r="K14" t="str">
+        <x:v>悉尼冬季晴天概率较好，早晚凉。</x:v>
+      </x:c>
+      <x:c r="L14" t="str">
+        <x:v>薄羽绒或风衣，海港边风大时注意保暖。</x:v>
+      </x:c>
+      <x:c r="M14" t="str">
+        <x:v>/itinerary/d12-sydney-opera-garden.png</x:v>
+      </x:c>
+      <x:c r="N14" t="str">
+        <x:v>悉尼歌剧院与植物园</x:v>
+      </x:c>
+      <x:c r="O14" t="str">
+        <x:v>步行 + 市内交通</x:v>
+      </x:c>
+      <x:c r="P14" t="str">
+        <x:v>08:45 前出门，09:15 前到 Sydney Opera House</x:v>
+      </x:c>
+      <x:c r="Q14" t="str">
+        <x:v>oaks-sydney-map</x:v>
+      </x:c>
+      <x:c r="R14" t="str">
+        <x:v>opera-house-map</x:v>
+      </x:c>
+      <x:c r="S14" t="str">
+        <x:v>opera-house-official</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d13</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D13</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-10</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周一</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悉尼南海岸</x:t>
-        </x:is>
+      <x:c r="A15" t="str">
+        <x:v>d13</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>D13</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>周一</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>悉尼南海岸</x:v>
       </x:c>
       <x:c r="F15" t="n">
         <x:v>-34.6713</x:v>
@@ -1853,92 +1421,58 @@
       <x:c r="G15" t="n">
         <x:v>150.8565</x:v>
       </x:c>
-      <x:c r="H15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">南海岸：Kiama、Gerringong 与袋鼠谷</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">沿 Grand Pacific Drive 南下，串联海崖桥与南海岸小镇。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Oaks Sydney Goldsbrough Suites</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">南海岸晴天最出片；沿海有风，袋鼠谷山区傍晚更凉。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">海边防风，穿舒适步行鞋；出发前检查 Royal National Park 道路警报。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/d13-south-coast-kiama-gerringong.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Kiama 与 Gerringong 南海岸公路</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">自驾（南海岸）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">08:00 出发；14:40 在 Gerringong 决定是否延伸袋鼠谷</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">oaks-sydney-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">sea-cliff-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">no-fixed-ticket</x:t>
-        </x:is>
+      <x:c r="H15" t="str">
+        <x:v>悉尼南海岸：Sea Cliff Bridge、Kiama 与 Gerringong</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>沿 Grand Pacific Drive 南下，经过 Sea Cliff Bridge、Kiama 与 Gerringong，视情况延伸袋鼠谷。</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>Oaks Sydney Goldsbrough Suites</x:v>
+      </x:c>
+      <x:c r="K15" t="str">
+        <x:v>南海岸晴天最出片；沿海有风，袋鼠谷山区傍晚更凉。</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>海边防风，穿舒适步行鞋；出发前检查 Royal National Park 道路警报。</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
+        <x:v>/itinerary/d13-south-coast-kiama-gerringong.png</x:v>
+      </x:c>
+      <x:c r="N15" t="str">
+        <x:v>Kiama 与 Gerringong 南海岸公路</x:v>
+      </x:c>
+      <x:c r="O15" t="str">
+        <x:v>自驾（南海岸）</x:v>
+      </x:c>
+      <x:c r="P15" t="str">
+        <x:v>08:00 出发；14:40 在 Gerringong 决定是否延伸袋鼠谷</x:v>
+      </x:c>
+      <x:c r="Q15" t="str">
+        <x:v>oaks-sydney-map</x:v>
+      </x:c>
+      <x:c r="R15" t="str">
+        <x:v>sea-cliff-map</x:v>
+      </x:c>
+      <x:c r="S15" t="str">
+        <x:v>no-fixed-ticket</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d14</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D14</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-11</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周二</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悉尼</x:t>
-        </x:is>
+      <x:c r="A16" t="str">
+        <x:v>d14</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>D14</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>周二</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>悉尼</x:v>
       </x:c>
       <x:c r="F16" t="n">
         <x:v>-33.8688</x:v>
@@ -1946,92 +1480,58 @@
       <x:c r="G16" t="n">
         <x:v>151.2093</x:v>
       </x:c>
-      <x:c r="H16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Taronga Zoo + Bondi + Totti’s</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">上午看澳洲动物，下午走 Bondi 海岸，晚上吃 Totti’s。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Oaks Sydney Goldsbrough Suites</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悉尼冬季早晚凉，渡轮甲板、动物园高处和 Bondi 海边都有风。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">穿舒适步行鞋，薄外套随身；Bondi 海岸步道只走短段。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/d14-taronga-bondi.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Taronga Zoo、悉尼港与 Bondi 海岸</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">F2 Ferry + 打车 / 市内交通 + 步行</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">08:30–09:00 出门前往 Circular Quay；18:15 前抵达 Totti’s</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">oaks-sydney-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">taronga-zoo-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">taronga-zoo-official</x:t>
-        </x:is>
+      <x:c r="H16" t="str">
+        <x:v>动物园到海岸：Taronga、Bondi 与 Totti’s</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>搭渡轮看 Taronga 的澳洲动物，下午走 Bondi 海岸，晚上在 Totti’s 用餐。</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>Oaks Sydney Goldsbrough Suites</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>悉尼冬季早晚凉，渡轮甲板、动物园高处和 Bondi 海边都有风。</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>穿舒适步行鞋，薄外套随身；Bondi 海岸步道只走短段。</x:v>
+      </x:c>
+      <x:c r="M16" t="str">
+        <x:v>/itinerary/d14-taronga-bondi.png</x:v>
+      </x:c>
+      <x:c r="N16" t="str">
+        <x:v>Taronga Zoo、悉尼港与 Bondi 海岸</x:v>
+      </x:c>
+      <x:c r="O16" t="str">
+        <x:v>F2 Ferry + 打车 / 市内交通 + 步行</x:v>
+      </x:c>
+      <x:c r="P16" t="str">
+        <x:v>08:30–09:00 出门前往 Circular Quay；18:15 前抵达 Totti’s</x:v>
+      </x:c>
+      <x:c r="Q16" t="str">
+        <x:v>oaks-sydney-map</x:v>
+      </x:c>
+      <x:c r="R16" t="str">
+        <x:v>taronga-zoo-map</x:v>
+      </x:c>
+      <x:c r="S16" t="str">
+        <x:v>taronga-zoo-official</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d15</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D15</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-12</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周三</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悉尼</x:t>
-        </x:is>
+      <x:c r="A17" t="str">
+        <x:v>d15</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>D15</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>2026-08-12</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>周三</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>悉尼</x:v>
       </x:c>
       <x:c r="F17" t="n">
         <x:v>-33.8688</x:v>
@@ -2039,92 +1539,58 @@
       <x:c r="G17" t="n">
         <x:v>151.2093</x:v>
       </x:c>
-      <x:c r="H17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Manly 弹性早晨 + 最后采购 + Cafe Sydney</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">早上按状态决定 Manly，下午采购整理，傍晚 Cafe Sydney。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Oaks Sydney Goldsbrough Suites</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悉尼早晚凉，若去 Manly，渡轮甲板和海边风更明显。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">薄外套随身；晚餐换 smart casual，并给回酒店整理行李留足时间。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/d15-manly-flex-farewell.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Manly 渡轮与悉尼港告别黄昏</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">F1 Ferry（可选） + 步行 / 市内交通</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">上午按状态决定；去 Manly 则 13:00–13:30 返程；16:40 前往 Cafe Sydney</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">oaks-sydney-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">qvb-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">no-fixed-ticket</x:t>
-        </x:is>
+      <x:c r="H17" t="str">
+        <x:v>悉尼告别日：可选 Manly、最后采购与 Cafe Sydney</x:v>
+      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>上午悠闲安排 Manly 或 CBD，下午采购并整理行李，傍晚在 Cafe Sydney 告别。</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>Oaks Sydney Goldsbrough Suites</x:v>
+      </x:c>
+      <x:c r="K17" t="str">
+        <x:v>悉尼早晚凉，若去 Manly，渡轮甲板和海边风更明显。</x:v>
+      </x:c>
+      <x:c r="L17" t="str">
+        <x:v>薄外套随身；晚餐换 smart casual，并给回酒店整理行李留足时间。</x:v>
+      </x:c>
+      <x:c r="M17" t="str">
+        <x:v>/itinerary/d15-manly-flex-farewell.png</x:v>
+      </x:c>
+      <x:c r="N17" t="str">
+        <x:v>Manly 渡轮与悉尼港告别黄昏</x:v>
+      </x:c>
+      <x:c r="O17" t="str">
+        <x:v>F1 Ferry（可选） + 步行 / 市内交通</x:v>
+      </x:c>
+      <x:c r="P17" t="str">
+        <x:v>上午按状态决定；去 Manly 则 13:00–13:30 返程；16:40 前往 Cafe Sydney</x:v>
+      </x:c>
+      <x:c r="Q17" t="str">
+        <x:v>oaks-sydney-map</x:v>
+      </x:c>
+      <x:c r="R17" t="str">
+        <x:v>qvb-map</x:v>
+      </x:c>
+      <x:c r="S17" t="str">
+        <x:v>no-fixed-ticket</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">d16</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D16</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-08-13</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">周四</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">悉尼 → 香港 → 上海</x:t>
-        </x:is>
+      <x:c r="A18" t="str">
+        <x:v>d16</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>D16</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>2026-08-13</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>周四</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>悉尼 → 香港 → 上海</x:v>
       </x:c>
       <x:c r="F18" t="n">
         <x:v>-33.9399</x:v>
@@ -2132,65 +1598,41 @@
       <x:c r="G18" t="n">
         <x:v>151.1753</x:v>
       </x:c>
-      <x:c r="H18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">返程与 TRS 退税</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">完成 TRS 与机场手续，启程回家。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">-</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">机场和机舱温差明显。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">提前整理退税物品和购物小票，随身带薄外套。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">/itinerary/d16-return-flight.png</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">澳洲旅行返程</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">航班 / 机场转场</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">按国际航班时间倒推，提前 3 小时到悉尼机场</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">sydney-airport-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">sydney-airport-map</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">trs-official</x:t>
-        </x:is>
+      <x:c r="H18" t="str">
+        <x:v>告别澳洲：TRS 退税与返程</x:v>
+      </x:c>
+      <x:c r="I18" t="str">
+        <x:v>完成 TRS 与机场手续，带着旅程回家。</x:v>
+      </x:c>
+      <x:c r="J18" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="K18" t="str">
+        <x:v>机场和机舱温差明显。</x:v>
+      </x:c>
+      <x:c r="L18" t="str">
+        <x:v>提前整理退税物品和购物小票，随身带薄外套。</x:v>
+      </x:c>
+      <x:c r="M18" t="str">
+        <x:v>/itinerary/d16-return-flight.png</x:v>
+      </x:c>
+      <x:c r="N18" t="str">
+        <x:v>澳洲旅行返程</x:v>
+      </x:c>
+      <x:c r="O18" t="str">
+        <x:v>航班 / 机场转场</x:v>
+      </x:c>
+      <x:c r="P18" t="str">
+        <x:v>按国际航班时间倒推，提前 3 小时到悉尼机场</x:v>
+      </x:c>
+      <x:c r="Q18" t="str">
+        <x:v>sydney-airport-map</x:v>
+      </x:c>
+      <x:c r="R18" t="str">
+        <x:v>sydney-airport-map</x:v>
+      </x:c>
+      <x:c r="S18" t="str">
+        <x:v>trs-official</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2258,7 +1700,7 @@
         <x:v>旅程开始</x:v>
       </x:c>
       <x:c r="G2" t="str">
-        <x:v>护照、签证、酒店信息和第一晚随身物品放随身包</x:v>
+        <x:v>护照、签证、酒店信息和抵达墨尔本后的随身用品放在随身包。</x:v>
       </x:c>
       <x:c r="H2" t="str">
         <x:v>flight-cathay</x:v>
@@ -2284,7 +1726,7 @@
         <x:v>初到澳洲，适应南半球冬天</x:v>
       </x:c>
       <x:c r="G3" t="str">
-        <x:v>4人 + 行李较多，打车 / Uber 更舒服；拍照：机场到达、第一眼 Melbourne CBD</x:v>
+        <x:v>4 人加行李较多，打车 / Uber 更舒服；从机场到 CBD 的沿途就是旅程的第一眼。</x:v>
       </x:c>
       <x:c r="H3" t="str">
         <x:v>mel-airport-map</x:v>
@@ -2310,7 +1752,7 @@
         <x:v>墨尔本咖啡文化开场</x:v>
       </x:c>
       <x:c r="G4" t="str">
-        <x:v>不要急着暴走，先恢复；拍照：咖啡桌面、街角 café</x:v>
+        <x:v>先寄存行李，找一家街角 café 吃早餐，让身体慢慢进入墨尔本节奏。</x:v>
       </x:c>
       <x:c r="H4" t="str">
         <x:v>oaks-market-map,oaks-market-booking,operator25-map</x:v>
@@ -2336,7 +1778,7 @@
         <x:v>墨尔本巷弄文化</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>如果疲惫，就只做 Degraves + Flinders，不再加远点；拍照：Degraves Street 巷道纵深、Flinders Street Station 外观</x:v>
+        <x:v>体力一般时走 Degraves Lane 与 Flinders Street 已经很充实；有余力再继续。</x:v>
       </x:c>
       <x:c r="H5" t="str">
         <x:v>degraves-map,flinders-street-map</x:v>
@@ -2362,7 +1804,7 @@
         <x:v>历史建筑 + 圆顶阅览室</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>只短暂停留拍照，不必完整逛；拍照：State Library 圆顶阅览室 6F 俯拍</x:v>
+        <x:v>在圆顶阅览室停留片刻即可，六楼俯拍视角最完整。</x:v>
       </x:c>
       <x:c r="H6" t="str">
         <x:v>state-library-map</x:v>
@@ -2388,7 +1830,7 @@
         <x:v>墨尔本意大利移民街区 + café culture</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>固定站点，控制在 60–90 分钟；若当天延误，先删 NGV，不删 Carlton 或 QVM</x:v>
+        <x:v>建议预留 60–90 分钟，在 Lygon Street 喝咖啡或吃 gelato；抵达较晚时可略过 NGV。</x:v>
       </x:c>
       <x:c r="H7" t="str">
         <x:v>carlton-lygon-map</x:v>
@@ -2414,7 +1856,7 @@
         <x:v>街头艺术 + 文艺墨尔本</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>20-30 分钟足够；拍照：Hosier Lane 涂鸦墙主背景</x:v>
+        <x:v>预留 20–30 分钟，选一面喜欢的涂鸦墙慢慢拍。</x:v>
       </x:c>
       <x:c r="H8" t="str">
         <x:v>hosier-map</x:v>
@@ -2440,7 +1882,7 @@
         <x:v>冬天避风避寒</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>Carlton 为固定站点；若时间不足，先跳过 NGV；拍照：NGV 中庭 / 红幕布</x:v>
+        <x:v>天气冷或想在室内休息时再去；时间有限可直接前往 Carlton。</x:v>
       </x:c>
       <x:c r="H9" t="str">
         <x:v>ngv-map</x:v>
@@ -2466,7 +1908,7 @@
         <x:v>冬季周三限定夜市</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>官方场次 17:00-22:00，免费入场、免预约；落地日建议 17:30 前到，按体力逛 30-120 分钟，穿防风保暖外套。</x:v>
+        <x:v>开放时间 17:00-22:00，免费入场、免预约；建议 17:30 左右到，按体力逛 30–120 分钟。</x:v>
       </x:c>
       <x:c r="H10" t="str">
         <x:v>qvm-map,qvm-winter-night-market-official</x:v>
@@ -2492,7 +1934,7 @@
         <x:v>落地日收尾</x:v>
       </x:c>
       <x:c r="G11" t="str">
-        <x:v>不再另订正式餐厅；如体力不足，可只逛 30-60 分钟后返回酒店。</x:v>
+        <x:v>在夜市吃过晚餐就回酒店休息；体力有限时逛 30–60 分钟也很合适。</x:v>
       </x:c>
       <x:c r="H11" t="str">
         <x:v>qvm-map,oaks-market-map,qvm-winter-night-market-official</x:v>
@@ -2515,10 +1957,10 @@
         <x:v>早餐：CBD café / Operator25（可选 Brunch）；午餐：Degraves Lane / CBD 简餐 / Pho Tùng（可选）；Carlton：咖啡或 gelato；晚餐：QVM Winter Night Market 街头热食（主）/ CBD 简餐（体力不足）</x:v>
       </x:c>
       <x:c r="F12" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G12" t="str">
-        <x:v>Carlton 只做轻量 café / gelato；QVM 夜市仍作为晚餐，不再另排 Southbank 正式晚餐。</x:v>
+        <x:v>Carlton 适合用一杯咖啡或 gelato 稍作休息；晚餐就在 QVM 冬季夜市边逛边吃。</x:v>
       </x:c>
       <x:c r="H12" t="str">
         <x:v>qvm-map,qvm-winter-night-market-official,operator25-map,pho-tung-map,degraves-map</x:v>
@@ -2648,7 +2090,7 @@
         <x:v>湖边公园、游客中心、火车站台氛围</x:v>
       </x:c>
       <x:c r="G17" t="str">
-        <x:v>不安排正式深度游，轻松走走即可</x:v>
+        <x:v>沿湖边和游客中心轻松走走，留出返程时间。</x:v>
       </x:c>
       <x:c r="H17" t="str">
         <x:v>emerald-lake-park-map,lakeside-station-map</x:v>
@@ -2674,7 +2116,7 @@
         <x:v>茶屋、糖果店、Dandenong Ranges 小镇感</x:v>
       </x:c>
       <x:c r="G18" t="str">
-        <x:v>只做短停，不安排正式下午茶，避免拖慢行程</x:v>
+        <x:v>逛一两家小店、喝杯热饮即可，注意返程集合时间。</x:v>
       </x:c>
       <x:c r="H18" t="str">
         <x:v>sassafras-map</x:v>
@@ -2697,7 +2139,7 @@
         <x:v>半日团结束，回到 CBD</x:v>
       </x:c>
       <x:c r="F19" t="str">
-        <x:v>时间较早，下午还能补一点市区内容</x:v>
+        <x:v>返城后继续 Fitzroy 街区漫步</x:v>
       </x:c>
       <x:c r="G19" t="str">
         <x:v>半日团结束后直接前往 Fitzroy；保持约 90 分钟街区时间</x:v>
@@ -2726,7 +2168,7 @@
         <x:v>街头艺术、老建筑与本地生活版墨尔本</x:v>
       </x:c>
       <x:c r="G20" t="str">
-        <x:v>固定站点，控制约 90 分钟；18:00 左右离开并回酒店整理大洋路行李</x:v>
+        <x:v>预留约 90 分钟，从 Brunswick Street 走到 Gertrude Street；18:00 左右回酒店整理行李。</x:v>
       </x:c>
       <x:c r="H20" t="str">
         <x:v>fitzroy-map,russell-343-map</x:v>
@@ -2749,7 +2191,7 @@
         <x:v>简单晚餐 + 整理大洋路行李</x:v>
       </x:c>
       <x:c r="F21" t="str">
-        <x:v>为 D3 机场取车做准备</x:v>
+        <x:v>为次日大洋路做好准备</x:v>
       </x:c>
       <x:c r="G21" t="str">
         <x:v>大件行李寄存，只带登机箱和随身包上大洋路；早点睡</x:v>
@@ -2775,10 +2217,10 @@
         <x:v>早餐：酒店附近 café / 集合前简单吃；午餐：Lakeside / Emerald Lake Park café 或团中简餐；晚餐：CBD / Southbank 轻松晚餐</x:v>
       </x:c>
       <x:c r="F22" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G22" t="str">
-        <x:v>半日团当天不安排升级餐厅，重点是准时集合和晚上整理行李</x:v>
+        <x:v>集合前吃得简单些；返城后在 Fitzroy / CBD 轻松晚餐，留出整理行李的时间。</x:v>
       </x:c>
       <x:c r="H22" t="str">
         <x:v>russell-343-map,emerald-lake-park-map,sassafras-map,southbank-map</x:v>
@@ -2801,10 +2243,10 @@
         <x:v>前往机场取车，确认车辆、保险、第二驾驶人、导航和行李安排</x:v>
       </x:c>
       <x:c r="F23" t="str">
-        <x:v>Road trip 正式开始</x:v>
+        <x:v>从机场取车，正式驶上大洋路</x:v>
       </x:c>
       <x:c r="G23" t="str">
-        <x:v>不在 CBD 内取车，降低右舵第一天压力；取车后先设置好导航和语音提示</x:v>
+        <x:v>从机场取车能避开 CBD 复杂路况；出发前先设置导航和语音提示，让右舵适应更从容。</x:v>
       </x:c>
       <x:c r="H23" t="str">
         <x:v>mel-airport-map</x:v>
@@ -2830,7 +2272,7 @@
         <x:v>右舵适应第一段</x:v>
       </x:c>
       <x:c r="G24" t="str">
-        <x:v>经过 Geelong 外围即可，不进 Geelong 市区；第一段以安全和适应为主</x:v>
+        <x:v>经过 Geelong 外围即可，刚开始适应右舵时把安全放在第一位。</x:v>
       </x:c>
       <x:c r="H24" t="str">
         <x:v>mel-airport-map,torquay-map</x:v>
@@ -2856,7 +2298,7 @@
         <x:v>大洋路氛围开始</x:v>
       </x:c>
       <x:c r="G25" t="str">
-        <x:v>Torquay 可作为第一正式休息点，不要一开始就频繁停车</x:v>
+        <x:v>把 Torquay 作为第一处完整休息点，喝杯咖啡再进入海岸线。</x:v>
       </x:c>
       <x:c r="H25" t="str">
         <x:v>torquay-map</x:v>
@@ -2986,7 +2428,7 @@
         <x:v>最舒服海滨小镇之一</x:v>
       </x:c>
       <x:c r="G30" t="str">
-        <x:v>今天真正的休息点放在 Lorne，不赶</x:v>
+        <x:v>在 Lorne 慢慢吃午餐、补给并休息，不必赶时间。</x:v>
       </x:c>
       <x:c r="H30" t="str">
         <x:v>lorne-map</x:v>
@@ -3116,7 +2558,7 @@
         <x:v>海边渔港氛围</x:v>
       </x:c>
       <x:c r="G35" t="str">
-        <x:v>D3 不做饭，轻松吃 fish &amp; chips / 海鲜，早点休息</x:v>
+        <x:v>到 Apollo Bay 后吃 fish &amp; chips 或海鲜，早点休息。</x:v>
       </x:c>
       <x:c r="H35" t="str">
         <x:v>apollo-map,fishermens-coop-map</x:v>
@@ -3139,10 +2581,10 @@
         <x:v>早餐：出发咖啡；午餐：Lorne café / Snow Monkey Ramen（备选）；晚餐：Apollo Bay Fishermen’s Co-op / seafood café</x:v>
       </x:c>
       <x:c r="F36" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G36" t="str">
-        <x:v>第一天右舵 + 海岸驾驶，不折腾做饭；fish &amp; chips / 海鲜最适合</x:v>
+        <x:v>海岸驾驶日以轻松好吃为主，Apollo Bay 的 fish &amp; chips / 海鲜正合适。</x:v>
       </x:c>
       <x:c r="H36" t="str">
         <x:v>lorne-map,snow-monkey-ramen-map,apollo-map,fishermens-coop-map</x:v>
@@ -3217,7 +2659,7 @@
         <x:v>十二使徒岩主观景台</x:v>
       </x:c>
       <x:c r="F39" t="str">
-        <x:v>世界级海岸地貌，大洋路地标</x:v>
+        <x:v>大洋路最具代表性的海岸地貌</x:v>
       </x:c>
       <x:c r="G39" t="str">
         <x:v>左侧平台更适合拍海岸线纵深；如果人多，不要停太久</x:v>
@@ -3243,7 +2685,7 @@
         <x:v>峡谷、海湾、海蚀地貌</x:v>
       </x:c>
       <x:c r="F40" t="str">
-        <x:v>D4 核心拍摄点，比十二使徒更值得慢慢看</x:v>
+        <x:v>峡谷、海湾与沉船海岸故事</x:v>
       </x:c>
       <x:c r="G40" t="str">
         <x:v>这里要认真留时间，不要只拍一张就走</x:v>
@@ -3344,13 +2786,13 @@
         <x:v>Port Campbell</x:v>
       </x:c>
       <x:c r="E44" t="str">
-        <x:v>买食材后视情况决定：附近 public electric BBQ / villa 厨房自炊 / 外食备选</x:v>
+        <x:v>抵达后按天气选择公共电烤炉 BBQ、villa 厨房自炊或附近餐厅</x:v>
       </x:c>
       <x:c r="F44" t="str">
         <x:v>灵活完成 BBQ-style dinner</x:v>
       </x:c>
       <x:c r="G44" t="str">
-        <x:v>Southern Ocean Villas 不提供自有 BBQ，但附近有两个免费 electric BBQ；villa 厨房完整，提供油、盐、胡椒和锡纸</x:v>
+        <x:v>Southern Ocean Villas 没有自带 BBQ，但附近有两处免费 electric BBQ；villa 厨房备有油、盐、胡椒和锡纸。</x:v>
       </x:c>
       <x:c r="H44" t="str">
         <x:v>port-campbell-map</x:v>
@@ -3370,13 +2812,13 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E45" t="str">
-        <x:v>早餐：Apollo Bay café；午餐：轻食 / picnic；晚餐：Apollo Bay 主采购食材 → 抵达 Southern Ocean Villas 后看天气和时间：可去附近 public electric BBQ；不行就 villa 厨房自炊</x:v>
+        <x:v>早餐：Apollo Bay café；午餐：轻食 / picnic；晚餐：在 Apollo Bay 买好食材，抵达后按天气选择公共 electric BBQ 或 villa 厨房自炊</x:v>
       </x:c>
       <x:c r="F45" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G45" t="str">
-        <x:v>不把 Port Campbell 当主采购点；核心是 BBQ-style dinner，不强求户外；villa 有完整厨房、锅具、餐具、油盐胡椒和锡纸</x:v>
+        <x:v>食材尽量在 Apollo Bay 买齐；抵达后视天气选择公共 BBQ 或 villa 厨房。</x:v>
       </x:c>
       <x:c r="H45" t="str">
         <x:v>apollo-map,port-campbell-map</x:v>
@@ -3396,13 +2838,13 @@
         <x:v>Twelve Apostles / Loch Ard Gorge</x:v>
       </x:c>
       <x:c r="E46" t="str">
-        <x:v>清晨补拍</x:v>
+        <x:v>清晨再看一处海岸景点</x:v>
       </x:c>
       <x:c r="F46" t="str">
         <x:v>光线柔和，人相对少</x:v>
       </x:c>
       <x:c r="G46" t="str">
-        <x:v>如果 D4 天气不好，这天可补救；二选一即可，不必两个都重刷</x:v>
+        <x:v>若前一天下雨，可在十二使徒岩或 Loch Ard Gorge 中选一处重访；天气好则按时间择一。</x:v>
       </x:c>
       <x:c r="H46" t="str">
         <x:v>twelve-apostles-map,loch-ard-map</x:v>
@@ -3500,7 +2942,7 @@
         <x:v>Bay of Islands</x:v>
       </x:c>
       <x:c r="E50" t="str">
-        <x:v>可选加点</x:v>
+        <x:v>时间充裕时延伸</x:v>
       </x:c>
       <x:c r="F50" t="str">
         <x:v>更开阔、更荒凉的海蚀柱群</x:v>
@@ -3555,7 +2997,7 @@
         <x:v>抵达机场、还车、取回寄存大件行李</x:v>
       </x:c>
       <x:c r="F52" t="str">
-        <x:v>Road trip 收束</x:v>
+        <x:v>大洋路自驾收尾</x:v>
       </x:c>
       <x:c r="G52" t="str">
         <x:v>预留加油、找还车点、整理车内物品和取行李时间</x:v>
@@ -3604,13 +3046,13 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E54" t="str">
-        <x:v>早餐：Port Campbell café；午餐：Colac / Timboon Ice Cream（🔥）；晚餐：机场酒店简餐</x:v>
+        <x:v>早餐：Port Campbell café；午餐：Colac / Timboon Ice Cream；晚餐：机场酒店简餐</x:v>
       </x:c>
       <x:c r="F54" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G54" t="str">
-        <x:v>冰淇淋补偿日；晚餐不折腾，重点是还车、取行李、整理热带段</x:v>
+        <x:v>Timboon Ice Cream 可作为回程中的小惊喜；抵达机场后简单用餐并整理行李。</x:v>
       </x:c>
       <x:c r="H54" t="str">
         <x:v>colac-map,timboon-icecream-map,port-campbell-map,holiday-inn-airport-map</x:v>
@@ -3712,7 +3154,7 @@
         <x:v>热闹轻松</x:v>
       </x:c>
       <x:c r="G58" t="str">
-        <x:v>今日不安排正式大餐</x:v>
+        <x:v>在夜市边逛边吃，让转场日轻松收尾。</x:v>
       </x:c>
       <x:c r="H58" t="str">
         <x:v>cairns-night-market-map</x:v>
@@ -3732,13 +3174,13 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E59" t="str">
-        <x:v>早餐：飞机/机场；午餐：简餐 / overlay coffee（花生拿铁🔥）；晚餐：Night Market</x:v>
+        <x:v>早餐：飞机 / 机场；午餐：简餐 / Overlay Coffee（可试花生拿铁）；晚餐：Cairns Night Markets</x:v>
       </x:c>
       <x:c r="F59" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G59" t="str">
-        <x:v>花生咖啡可试</x:v>
+        <x:v>到凯恩斯后的第一杯可以试试花生咖啡，晚上随意逛夜市。</x:v>
       </x:c>
       <x:c r="H59"/>
     </x:row>
@@ -3840,7 +3282,7 @@
         <x:v>通常会比较疲惫</x:v>
       </x:c>
       <x:c r="G63" t="str">
-        <x:v>晚上不要订太正式的餐厅</x:v>
+        <x:v>下船后回酒店休息，晚间只留一顿轻松晚餐。</x:v>
       </x:c>
       <x:c r="H63" t="str">
         <x:v>reef-fleet-terminal-map</x:v>
@@ -3866,7 +3308,7 @@
         <x:v>海边晚餐</x:v>
       </x:c>
       <x:c r="G64" t="str">
-        <x:v>轻松即可，不要再安排夜间项目</x:v>
+        <x:v>按体力选码头附近餐厅，轻松吃完就回酒店。</x:v>
       </x:c>
       <x:c r="H64" t="str">
         <x:v>prawn-star-map,salt-house-map,dundees-map</x:v>
@@ -3886,13 +3328,13 @@
         <x:v>今日提醒</x:v>
       </x:c>
       <x:c r="E65" t="str">
-        <x:v>Reef Magic 是凯恩斯段核心项目，重点是完成一次稳定的大堡礁外礁体验。</x:v>
+        <x:v>Reef Magic 是今天的主角，先照顾好海况、晕船和体力，再慢慢享受外礁。</x:v>
       </x:c>
       <x:c r="F65" t="str">
-        <x:v>海况、风浪、晕船和体力比晴雨更影响体验</x:v>
+        <x:v>舒适与安全比拍摄数量更重要</x:v>
       </x:c>
       <x:c r="G65" t="str">
-        <x:v>不必追求拍很多水下画面，先保证舒适和安全。</x:v>
+        <x:v>水下照片随缘，先保证自己舒服、安全。</x:v>
       </x:c>
       <x:c r="H65" t="str">
         <x:v>reef-magic-official</x:v>
@@ -3915,10 +3357,10 @@
         <x:v>早餐：酒店轻食；午餐：Reef Magic 外礁平台午餐（已订）；晚餐：Prawn Star / Salt House</x:v>
       </x:c>
       <x:c r="F66" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G66" t="str">
-        <x:v>出海后不要订太正式的餐厅，视体力轻松吃</x:v>
+        <x:v>出海回来通常会累，码头附近找一家顺眼的店轻松吃。</x:v>
       </x:c>
       <x:c r="H66" t="str">
         <x:v>reef-magic-official,prawn-star-map,salt-house-map</x:v>
@@ -4015,7 +3457,7 @@
         <x:v>雨林入海、海滩短停留</x:v>
       </x:c>
       <x:c r="F70" t="str">
-        <x:v>这天最特别的画面</x:v>
+        <x:v>雨林与海洋在这里交会</x:v>
       </x:c>
       <x:c r="G70" t="str">
         <x:v>不建议下海游泳；注意鳄鱼、水母和警示牌</x:v>
@@ -4041,7 +3483,7 @@
         <x:v>渡河、热带水果冰淇淋</x:v>
       </x:c>
       <x:c r="F71" t="str">
-        <x:v>Daintree Ice-Cream Company 是很强的 only here 体验</x:v>
+        <x:v>丹翠地区很有代表性的热带味道</x:v>
       </x:c>
       <x:c r="G71" t="str">
         <x:v>冰淇淋已包含在 Billy Tea 行程内</x:v>
@@ -4070,7 +3512,7 @@
         <x:v>回程可休息</x:v>
       </x:c>
       <x:c r="G72" t="str">
-        <x:v>晚餐简单，不再加夜间项目</x:v>
+        <x:v>回程车上可以休息，回到市区后就近吃晚餐。</x:v>
       </x:c>
       <x:c r="H72"/>
     </x:row>
@@ -4088,13 +3530,13 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E73" t="str">
-        <x:v>早餐：酒店早餐；午餐：团餐；晚餐：凯恩斯随便</x:v>
+        <x:v>早餐：酒店早餐；午餐：团餐；晚餐：凯恩斯市区简餐</x:v>
       </x:c>
       <x:c r="F73" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G73" t="str">
-        <x:v>Daintree Ice Cream 必吃；回程较晚，晚餐简单</x:v>
+        <x:v>团餐和热带水果冰淇淋都在行程里，回城较晚，晚餐简单即可。</x:v>
       </x:c>
       <x:c r="H73" t="str">
         <x:v>daintree-icecream-map</x:v>
@@ -4221,7 +3663,7 @@
         <x:v>瀑布短停留、拍照</x:v>
       </x:c>
       <x:c r="F78" t="str">
-        <x:v>阿瑟顿这一天的视觉高潮</x:v>
+        <x:v>雨林瀑布与高原绿意</x:v>
       </x:c>
       <x:c r="G78" t="str">
         <x:v>优先 Millaa Millaa；体力够再加 Ellinjaa，不必塞满全部瀑布</x:v>
@@ -4271,10 +3713,10 @@
         <x:v>简单晚餐</x:v>
       </x:c>
       <x:c r="F80" t="str">
-        <x:v>不安排正式大餐</x:v>
+        <x:v>回城后轻松晚餐</x:v>
       </x:c>
       <x:c r="G80" t="str">
-        <x:v>为周五休息日保留体力</x:v>
+        <x:v>下山后就近用餐，早点休息。</x:v>
       </x:c>
       <x:c r="H80"/>
     </x:row>
@@ -4292,13 +3734,13 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>早餐：café 早餐；午餐：Gallo Dairyland / Millaa Millaa；晚餐：回凯恩斯随便</x:v>
+        <x:v>早餐：café 早餐；午餐：Gallo Dairyland / Millaa Millaa；晚餐：凯恩斯市区简餐</x:v>
       </x:c>
       <x:c r="F81" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G81" t="str">
-        <x:v>奶制品 + 瀑布</x:v>
+        <x:v>午餐在高原小镇慢慢吃，回凯恩斯后按体力选一顿轻松晚餐。</x:v>
       </x:c>
       <x:c r="H81" t="str">
         <x:v>millaa-map,gallo-map</x:v>
@@ -4324,7 +3766,7 @@
         <x:v>周五正好开市，适合补水果和轻食</x:v>
       </x:c>
       <x:c r="G82" t="str">
-        <x:v>买能当天吃完或带上飞机前吃完的，不要买太多</x:v>
+        <x:v>优先买当天能吃完的水果与轻食，方便次日早班机。</x:v>
       </x:c>
       <x:c r="H82" t="str">
         <x:v>rustys-map</x:v>
@@ -4350,7 +3792,7 @@
         <x:v>热带城市躺平感</x:v>
       </x:c>
       <x:c r="G83" t="str">
-        <x:v>不安排远距离移动</x:v>
+        <x:v>午间留在酒店或 Esplanade 放松，让节奏慢下来。</x:v>
       </x:c>
       <x:c r="H83" t="str">
         <x:v>cairns-lagoon-map</x:v>
@@ -4400,7 +3842,7 @@
         <x:v>热带海滨小镇与凯恩斯北部海岸</x:v>
       </x:c>
       <x:c r="G85" t="str">
-        <x:v>固定站点，傍晚返回凯恩斯；不再叠加 Cairns Aquarium 或 Esplanade 长走</x:v>
+        <x:v>沿棕榈树海滨大道散步、喝杯咖啡，天黑前后返回凯恩斯。</x:v>
       </x:c>
       <x:c r="H85" t="str">
         <x:v>palm-cove-map</x:v>
@@ -4449,10 +3891,10 @@
         <x:v>早餐：Rusty’s Market / Market水果；午餐：简餐；晚餐：Prawn Star / seafood café（优先）</x:v>
       </x:c>
       <x:c r="F87" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G87" t="str">
-        <x:v>修复 + 海鲜；不要再加长线</x:v>
+        <x:v>Market 水果、海鲜和 Palm Cove 咖啡串成轻松的一天。</x:v>
       </x:c>
       <x:c r="H87" t="str">
         <x:v>rustys-map,prawn-star-map</x:v>
@@ -4475,7 +3917,7 @@
         <x:v>早起退房，打车 / Uber 前往机场</x:v>
       </x:c>
       <x:c r="F88" t="str">
-        <x:v>转场日开始</x:v>
+        <x:v>从凯恩斯启程前往悉尼</x:v>
       </x:c>
       <x:c r="G88" t="str">
         <x:v>前一晚必须完成打包；Jetstar 行李按 20kg 控制</x:v>
@@ -4551,10 +3993,10 @@
         <x:v>轻松适应，简单午餐或休息</x:v>
       </x:c>
       <x:c r="F91" t="str">
-        <x:v>不硬玩，恢复清晨航班疲劳</x:v>
+        <x:v>在 Darling Harbour 缓一缓</x:v>
       </x:c>
       <x:c r="G91" t="str">
-        <x:v>可在酒店附近熟悉环境</x:v>
+        <x:v>先休息、吃点东西，再开始海港散步。</x:v>
       </x:c>
       <x:c r="H91" t="str">
         <x:v>darling-harbour-map</x:v>
@@ -4580,7 +4022,7 @@
         <x:v>原生植物、砂岩海岸与悉尼港步行线</x:v>
       </x:c>
       <x:c r="G92" t="str">
-        <x:v>固定站点，控制约 45–60 分钟；转场日保持轻量，不增加收费项目</x:v>
+        <x:v>预留 45–60 分钟沿海滨慢慢走，转场日下午以看景和恢复为主。</x:v>
       </x:c>
       <x:c r="H92" t="str">
         <x:v>barangaroo-reserve-map,darling-harbour-map,the-rocks-map</x:v>
@@ -4603,10 +4045,10 @@
         <x:v>岩石区散步、晚餐</x:v>
       </x:c>
       <x:c r="F93" t="str">
-        <x:v>砂岩建筑、老城氛围</x:v>
+        <x:v>砂岩老街与海港傍晚</x:v>
       </x:c>
       <x:c r="G93" t="str">
-        <x:v>悉尼第一晚很适合这里</x:v>
+        <x:v>在 The Rocks 边走边找晚餐，感受悉尼老城区的第一晚。</x:v>
       </x:c>
       <x:c r="H93" t="str">
         <x:v>the-rocks-map</x:v>
@@ -4632,7 +4074,7 @@
         <x:v>悉尼开场画面</x:v>
       </x:c>
       <x:c r="G94" t="str">
-        <x:v>轻松看夜景即可，不要安排太复杂</x:v>
+        <x:v>看完歌剧院与海港大桥夜景后轻松回酒店。</x:v>
       </x:c>
       <x:c r="H94" t="str">
         <x:v>circular-quay-map</x:v>
@@ -4655,10 +4097,10 @@
         <x:v>早餐：café / A.P Bakery（可选）；午餐：飞机/机场 / mezze feast；晚餐：The Rocks pub</x:v>
       </x:c>
       <x:c r="F95" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G95" t="str">
-        <x:v>转场日，晚餐轻松</x:v>
+        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
       </x:c>
       <x:c r="H95" t="str">
         <x:v>the-rocks-map</x:v>
@@ -4840,7 +4282,7 @@
         <x:v>海港景观非常好</x:v>
       </x:c>
       <x:c r="G102" t="str">
-        <x:v>这段不是赶景点，是慢慢走向 Mrs Macquarie’s Chair；可拍草坪远景框住歌剧院 + 海港桥</x:v>
+        <x:v>沿海港步道慢慢走向 Mrs Macquarie’s Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
       </x:c>
       <x:c r="H102" t="str">
         <x:v>botanic-garden-map</x:v>
@@ -4918,7 +4360,7 @@
         <x:v>城市核心日收尾</x:v>
       </x:c>
       <x:c r="G105" t="str">
-        <x:v>不一定要升级晚餐，给 D14 / D15 留空间；达令港夜景可选</x:v>
+        <x:v>在 CBD / Darling Harbour 轻松收尾；达令港夜景按体力决定。</x:v>
       </x:c>
       <x:c r="H105" t="str">
         <x:v>darling-harbour-map,hello-auntie-map</x:v>
@@ -4941,10 +4383,10 @@
         <x:v>早餐：bills / Toby’s Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
       </x:c>
       <x:c r="F106" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G106" t="str">
-        <x:v>9:30 歌剧院中文导览已订；导览后固定步行前往 The Rocks Weekend Market，停留约 45–60 分钟</x:v>
+        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
       </x:c>
       <x:c r="H106" t="str">
         <x:v>bills-sydney-map,tobys-estate-map,the-rocks-map,the-rocks-market-official,circular-quay-map,hello-auntie-map</x:v>
@@ -4970,7 +4412,7 @@
         <x:v>城市切换到南海岸</x:v>
       </x:c>
       <x:c r="G107" t="str">
-        <x:v>路线已确定为南海岸；出发前查看 Royal National Park alerts，遇关闭按导航绕行</x:v>
+        <x:v>出发前查看 Royal National Park alerts，遇临时关闭按导航绕行。</x:v>
       </x:c>
       <x:c r="H107" t="str">
         <x:v>royal-national-park-map,bald-hill-map</x:v>
@@ -5048,7 +4490,7 @@
         <x:v>为 Kiama 留出完整窗口</x:v>
       </x:c>
       <x:c r="G110" t="str">
-        <x:v>不把 Wollongong 做成长停；进度慢就直接去 Kiama</x:v>
+        <x:v>在 Wollongong 喝杯咖啡即可，把完整午餐和散步留给 Kiama。</x:v>
       </x:c>
       <x:c r="H110" t="str">
         <x:v>wollongong-map</x:v>
@@ -5126,7 +4568,7 @@
         <x:v>海岸逐渐转为农场与小镇</x:v>
       </x:c>
       <x:c r="G113" t="str">
-        <x:v>Gerringong 距 Kiama 很近，是今天的确定停靠</x:v>
+        <x:v>从 Kiama 很快就能到 Gerringong，沿海公路和农场景色会自然切换。</x:v>
       </x:c>
       <x:c r="H113" t="str">
         <x:v>kiama-map,gerringong-map</x:v>
@@ -5152,7 +4594,7 @@
         <x:v>南海岸与乡村景观同框</x:v>
       </x:c>
       <x:c r="G114" t="str">
-        <x:v>不要在这里拖成完整下午；14:40 左右做袋鼠谷判断</x:v>
+        <x:v>预留约 55 分钟看海、喝咖啡；14:40 左右再决定是否前往袋鼠谷。</x:v>
       </x:c>
       <x:c r="H114" t="str">
         <x:v>gerringong-map</x:v>
@@ -5204,7 +4646,7 @@
         <x:v>海岸日的乡村加餐</x:v>
       </x:c>
       <x:c r="G116" t="str">
-        <x:v>只做 Hampden Bridge + 小镇短停；不再加 Fitzroy Falls</x:v>
+        <x:v>若前往袋鼠谷，只安排 Hampden Bridge 与小镇短停，16:15 前返程。</x:v>
       </x:c>
       <x:c r="H116" t="str">
         <x:v>kangaroo-valley-map,hampden-bridge-map</x:v>
@@ -5253,10 +4695,10 @@
         <x:v>早餐：café；午餐：Kiama Hungry Monkey / Kiama 简餐；晚餐：回城后 CBD / 酒店附近简餐</x:v>
       </x:c>
       <x:c r="F118" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G118" t="str">
-        <x:v>今天以南海岸驾驶为主；不为餐厅绕路，给 Gerringong 和可选袋鼠谷留时间</x:v>
+        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
       </x:c>
       <x:c r="H118" t="str">
         <x:v>kiama-map,kiama-hungry-monkey-map,gerringong-map,oaks-sydney-map</x:v>
@@ -5334,7 +4776,7 @@
         <x:v>澳洲本土动物 + Harbour view</x:v>
       </x:c>
       <x:c r="G121" t="str">
-        <x:v>不追求全园；当天动物展示和 keeper talk 以官网及现场为准</x:v>
+        <x:v>优先 Australian Wildlife 区域与海港景观，再按当天 keeper talk 调整顺序。</x:v>
       </x:c>
       <x:c r="H121" t="str">
         <x:v>taronga-zoo-map,taronga-zoo-official</x:v>
@@ -5386,7 +4828,7 @@
         <x:v>泳池、海浪、悬崖海岸线</x:v>
       </x:c>
       <x:c r="G123" t="str">
-        <x:v>不走完整 Bondi–Coogee；17:45 左右结束海边，给晚餐交通留时间</x:v>
+        <x:v>走 Bondi–Tamarama 短段即可，17:45 左右离开海边，从容前往晚餐。</x:v>
       </x:c>
       <x:c r="H123" t="str">
         <x:v>bondi-map,icebergs-map,tamarama-map</x:v>
@@ -5435,10 +4877,10 @@
         <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti’s Bondi 18:30（已订）</x:v>
       </x:c>
       <x:c r="F125" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G125" t="str">
-        <x:v>动物园午餐不要拖；下午只走 Bondi–Tamarama 短段，按时到 Totti’s</x:v>
+        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti’s。</x:v>
       </x:c>
       <x:c r="H125" t="str">
         <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
@@ -5458,13 +4900,13 @@
         <x:v>酒店 / 悉尼市区</x:v>
       </x:c>
       <x:c r="E126" t="str">
-        <x:v>慢早餐，按睡眠、天气和体力决定是否去 Manly</x:v>
+        <x:v>慢早餐，结合睡眠、天气和体力决定 Manly 或 CBD</x:v>
       </x:c>
       <x:c r="F126" t="str">
-        <x:v>最后一天保留弹性</x:v>
+        <x:v>告别日从容开场</x:v>
       </x:c>
       <x:c r="G126" t="str">
-        <x:v>状态好才启动 Manly；否则留在 CBD，直接进入轻松采购与整理</x:v>
+        <x:v>睡饱、天气好就去 Manly；否则留在 CBD 慢慢吃早餐。</x:v>
       </x:c>
       <x:c r="H126" t="str">
         <x:v>oaks-sydney-map,qvb-map</x:v>
@@ -5490,7 +4932,7 @@
         <x:v>悉尼港经典渡轮体验</x:v>
       </x:c>
       <x:c r="G127" t="str">
-        <x:v>仅在状态好且能于 13:00–13:30 返程时执行；当天查看班次</x:v>
+        <x:v>确认能在 13:00–13:30 前返程再出发，并查看当天船班。</x:v>
       </x:c>
       <x:c r="H127" t="str">
         <x:v>circular-quay-map,manly-ferry-map</x:v>
@@ -5516,7 +4958,7 @@
         <x:v>比 Bondi 更松弛</x:v>
       </x:c>
       <x:c r="G128" t="str">
-        <x:v>不追求打卡；午餐不要拖太久</x:v>
+        <x:v>在海边散步、喝咖啡，12:45 左右准备返程。</x:v>
       </x:c>
       <x:c r="H128" t="str">
         <x:v>manly-beach-map,hugos-manly-map,felons-manly-map</x:v>
@@ -5542,7 +4984,7 @@
         <x:v>给采购、TRS 和晚餐留余量</x:v>
       </x:c>
       <x:c r="G129" t="str">
-        <x:v>若早上没有去 Manly，这一时段可在 CBD 咖啡或提前购物</x:v>
+        <x:v>若上午留在 CBD，这段时间可喝咖啡或提前开始采购。</x:v>
       </x:c>
       <x:c r="H129" t="str">
         <x:v>manly-ferry-map,circular-quay-map,qvb-map</x:v>
@@ -5669,10 +5111,10 @@
         <x:v>早餐：café / Single O / Toby’s Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
       </x:c>
       <x:c r="F134" t="str">
-        <x:v>每日餐食参考</x:v>
+        <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G134" t="str">
-        <x:v>Manly 是状态触发项；无论去不去，14:00 后进入采购、TRS 和告别晚餐主线</x:v>
+        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
       </x:c>
       <x:c r="H134" t="str">
         <x:v>single-o-map,tobys-estate-map,manly-beach-map,qvb-map,cafe-sydney-map,cafe-sydney-official</x:v>
@@ -5692,13 +5134,13 @@
         <x:v>悉尼机场</x:v>
       </x:c>
       <x:c r="E135" t="str">
-        <x:v>办理 TRS 退税，登机返程。</x:v>
+        <x:v>办理 TRS 退税与登机手续，启程回家</x:v>
       </x:c>
       <x:c r="F135" t="str">
         <x:v>满载而归</x:v>
       </x:c>
       <x:c r="G135" t="str">
-        <x:v>提前下载 TRS App 填好信息，可走快速通道。</x:v>
+        <x:v>提前在 TRS App 填好信息，符合条件时可走快速通道。</x:v>
       </x:c>
       <x:c r="H135" t="str">
         <x:v>sydney-airport-map,trs-official</x:v>
@@ -5718,13 +5160,13 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E136" t="str">
-        <x:v>早餐：机场早餐；午餐：飞机；晚餐：无</x:v>
+        <x:v>早餐：机场早餐；午餐 / 晚餐：按航班餐食安排</x:v>
       </x:c>
       <x:c r="F136" t="str">
-        <x:v>无</x:v>
+        <x:v>返程日简单省心</x:v>
       </x:c>
       <x:c r="G136" t="str">
-        <x:v>结束</x:v>
+        <x:v>早点到机场，吃好早餐后按航班节奏休息。</x:v>
       </x:c>
       <x:c r="H136"/>
     </x:row>
@@ -8071,7 +7513,7 @@
         <x:v>no-fixed-ticket</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>当天无固定票券</x:v>
+        <x:v>今天无需提前购票</x:v>
       </x:c>
       <x:c r="C123" t="str">
         <x:v>note</x:v>
@@ -8080,7 +7522,7 @@
       <x:c r="E123"/>
       <x:c r="F123"/>
       <x:c r="G123" t="str">
-        <x:v>每日明确票券状态</x:v>
+        <x:v>当天以免费景点或灵活安排为主</x:v>
       </x:c>
     </x:row>
     <x:row r="124" s="23" customFormat="1" ht="30" customHeight="1">
@@ -9502,323 +8944,215 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D1 墨尔本</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">CBD café / Operator25（可选Brunch）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Degraves Lane / CBD 简餐 / Pho Tùng（可选）</x:t>
-        </x:is>
+      <x:c r="A2" t="str">
+        <x:v>D1 墨尔本</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>CBD café / Operator25（可选Brunch）</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>Degraves Lane / CBD 简餐 / Pho Tùng（可选）</x:v>
       </x:c>
       <x:c r="D2" t="str">
         <x:v>QVM Winter Night Market 街头热食（主）/ Carlton / Lygon Street café 或 gelato / CBD 简餐（体力不足）</x:v>
       </x:c>
       <x:c r="E2" t="str">
-        <x:v>Carlton / Little Italy 为固定站点；QVM 17:30-19:30 仍为周三限定主安排；延误时先删 NGV，不删 Carlton 或 QVM。</x:v>
+        <x:v>Carlton 适合用一杯咖啡或 gelato 稍作休息；晚餐就在 QVM 冬季夜市边逛边吃。</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D2 墨尔本 + Puffing Billy / Sassafras</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">酒店附近 café / 集合前简单吃</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Lakeside / Emerald Lake Park café 或团中简餐</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">CBD / Southbank 轻松晚餐</x:t>
-        </x:is>
+      <x:c r="A3" t="str">
+        <x:v>D2 墨尔本 + Puffing Billy / Sassafras</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>酒店附近 café / 集合前简单吃</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>Lakeside / Emerald Lake Park café 或团中简餐</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>CBD / Southbank 轻松晚餐</x:v>
       </x:c>
       <x:c r="E3" t="str">
-        <x:v>半日团返城后固定走 Fitzroy 约 90 分钟；随后回酒店整理大洋路行李</x:v>
+        <x:v>集合前吃得简单些；返城后在 Fitzroy / CBD 轻松晚餐，留出整理行李的时间。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D3 大洋路</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">出发咖啡</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Lorne café / Snow Monkey Ramen（备选）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Apollo Bay Fishermen’s Co-op / seafood café</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">第一天右舵 + 海岸驾驶，不折腾做饭；fish &amp; chips / 海鲜最适合</x:t>
-        </x:is>
+      <x:c r="A4" t="str">
+        <x:v>D3 大洋路</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>出发咖啡</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Lorne café / Snow Monkey Ramen（备选）</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Apollo Bay Fishermen’s Co-op / seafood café</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>海岸驾驶日以轻松好吃为主，Apollo Bay 的 fish &amp; chips / 海鲜正合适。</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D4 大洋路</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Apollo Bay café</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">轻食 / picnic</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Apollo Bay 主采购食材 → 抵达 Southern Ocean Villas 后看天气和时间：可去附近 public electric BBQ；不行就 villa 厨房自炊</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">不把 Port Campbell 当主采购点；核心是 BBQ-style dinner，不强求户外；villa 有完整厨房、锅具、餐具、油盐胡椒和锡纸</x:t>
-        </x:is>
+      <x:c r="A5" t="str">
+        <x:v>D4 大洋路</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Apollo Bay café</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>轻食 / picnic</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>Apollo Bay 主采购食材 → 抵达 Southern Ocean Villas 后看天气和时间：可去附近 public electric BBQ；不行就 villa 厨房自炊</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>食材尽量在 Apollo Bay 买齐；抵达后视天气选择公共 BBQ 或 villa 厨房。</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D5 回程</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Port Campbell café</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Colac / Timboon Ice Cream（🔥）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">机场酒店简餐</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E6" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">冰淇淋补偿日；晚餐不折腾，重点是还车、取行李、整理热带段</x:t>
-        </x:is>
+      <x:c r="A6" t="str">
+        <x:v>D5 回程</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Port Campbell café</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Colac / Timboon Ice Cream（🔥）</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>机场酒店简餐</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>Timboon Ice Cream 可作为回程中的小惊喜；抵达机场后简单用餐并整理行李。</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D6 凯恩斯</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">飞机/机场</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">简餐 / overlay coffee（花生拿铁🔥）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Night Market</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">花生咖啡可试</x:t>
-        </x:is>
+      <x:c r="A7" t="str">
+        <x:v>D6 凯恩斯</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>飞机/机场</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>简餐 / overlay coffee（花生拿铁🔥）</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>Night Market</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>到凯恩斯后的第一杯可以试试花生咖啡，晚上随意逛夜市。</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D7 大堡礁</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">酒店轻食</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Reef Magic 外礁平台午餐（已订）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Prawn Star / Salt House</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">出海后不要订太正式的餐厅，视体力轻松吃</x:t>
-        </x:is>
+      <x:c r="A8" t="str">
+        <x:v>D7 大堡礁</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>酒店轻食</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Reef Magic 外礁平台午餐（已订）</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>Prawn Star / Salt House</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>出海回来通常会累，码头附近找一家顺眼的店轻松吃。</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D8 丹翠</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">酒店早餐</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">团餐</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">凯恩斯随便</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Daintree Ice Cream 必吃；回程较晚，晚餐简单</x:t>
-        </x:is>
+      <x:c r="A9" t="str">
+        <x:v>D8 丹翠</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>酒店早餐</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>团餐</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>凯恩斯随便</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>团餐和热带水果冰淇淋都在行程里，回城较晚，晚餐简单即可。</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D9 阿瑟顿</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">café 早餐</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Gallo Dairyland / Millaa Millaa</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">回凯恩斯随便</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">奶制品 + 瀑布</x:t>
-        </x:is>
+      <x:c r="A10" t="str">
+        <x:v>D9 阿瑟顿</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>café 早餐</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>Gallo Dairyland / Millaa Millaa</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>回凯恩斯随便</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>午餐在高原小镇慢慢吃，回凯恩斯后按体力选一顿轻松晚餐。</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D10 凯恩斯</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Rusty’s Market / Market水果</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">简餐</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D11" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Prawn Star / seafood café（优先）</x:t>
-        </x:is>
+      <x:c r="A11" t="str">
+        <x:v>D10 凯恩斯</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>Rusty’s Market / Market水果</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>简餐</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>Prawn Star / seafood café（优先）</x:v>
       </x:c>
       <x:c r="E11" t="str">
-        <x:v>Rusty’s + 休息整理 + Palm Cove 固定半日；傍晚回凯恩斯，不再叠加长线</x:v>
+        <x:v>Market 水果、海鲜和 Palm Cove 咖啡串成轻松的一天。</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D11 悉尼</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">café / A.P Bakery（可选）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">飞机/机场 / mezze feast</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D12" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">The Rocks pub</x:t>
-        </x:is>
+      <x:c r="A12" t="str">
+        <x:v>D11 悉尼</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>café / A.P Bakery（可选）</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>飞机/机场 / mezze feast</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>The Rocks pub</x:v>
       </x:c>
       <x:c r="E12" t="str">
-        <x:v>转场日；酒店休息后固定经 Barangaroo Reserve / Wulugul Walk 前往 The Rocks 与 Circular Quay</x:v>
+        <x:v>转场日不赶餐厅，晚上在 The Rocks 找一家舒服的 pub 收尾。</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D12 悉尼</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bills / Toby’s Estate</x:t>
-        </x:is>
+      <x:c r="A13" t="str">
+        <x:v>D12 悉尼</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>bills / Toby’s Estate</x:v>
       </x:c>
       <x:c r="C13" t="str">
         <x:v>The Rocks Markets / Circular Quay 简餐</x:v>
       </x:c>
-      <x:c r="D13" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Hello Auntie</x:t>
-        </x:is>
+      <x:c r="D13" t="str">
+        <x:v>Hello Auntie</x:v>
       </x:c>
       <x:c r="E13" t="str">
-        <x:v>9:30 歌剧院中文导览已订；结束后步行前往 The Rocks Weekend Market，周日 10:00–17:00 开放，停留约 45–60 分钟；随后前往植物园和 QVB。</x:v>
+        <x:v>市集可边逛边吃；若只简单垫一口，晚上再去 Hello Auntie。</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
         <x:v>D13 南海岸</x:v>
       </x:c>
-      <x:c r="B14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">café</x:t>
-        </x:is>
+      <x:c r="B14" t="str">
+        <x:v>café</x:v>
       </x:c>
       <x:c r="C14" t="str">
         <x:v>Kiama Hungry Monkey / Kiama 简餐</x:v>
@@ -9827,17 +9161,15 @@
         <x:v>回城后 CBD / 酒店附近简餐</x:v>
       </x:c>
       <x:c r="E14" t="str">
-        <x:v>路线确定为 Sea Cliff Bridge + Kiama + Gerringong；Kangaroo Valley 视时间、天气和体力决定，不为餐厅绕路</x:v>
+        <x:v>午餐留在 Kiama，返城后就近用餐，把时间留给海岸和小镇。</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
         <x:v>D14 Taronga + Bondi</x:v>
       </x:c>
-      <x:c r="B15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">CBD café</x:t>
-        </x:is>
+      <x:c r="B15" t="str">
+        <x:v>CBD café</x:v>
       </x:c>
       <x:c r="C15" t="str">
         <x:v>Taronga Zoo 轻食 / Circular Quay 简餐</x:v>
@@ -9846,17 +9178,15 @@
         <x:v>Totti’s Bondi 18:30（已订）</x:v>
       </x:c>
       <x:c r="E15" t="str">
-        <x:v>上午动物园，下午 Bondi–Icebergs–Tamarama 短段；17:45 左右结束海边</x:v>
+        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti’s。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" s="23" customFormat="1" ht="40" customHeight="1">
       <x:c r="A16" s="25" t="str">
         <x:v>D15 Manly 弹性 + 告别</x:v>
       </x:c>
-      <x:c r="B16" s="25" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">café / Single O / Toby’s Estate</x:t>
-        </x:is>
+      <x:c r="B16" s="25" t="str">
+        <x:v>café / Single O / Toby’s Estate</x:v>
       </x:c>
       <x:c r="C16" s="25" t="str">
         <x:v>若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐</x:v>
@@ -9865,29 +9195,24 @@
         <x:v>Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
       </x:c>
       <x:c r="E16" s="25" t="str">
-        <x:v>早上看状态决定 Manly；14:00 后固定采购、TRS / 行李整理与告别晚餐</x:v>
+        <x:v>无论上午在哪，14:00 后都回到 CBD 采购、整理 TRS，最后去 Cafe Sydney。</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D16 返程</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">机场早餐</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">飞机</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D17" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">无</x:t>
-        </x:is>
+      <x:c r="A17" t="str">
+        <x:v>D16 返程</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>机场早餐</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>按航班餐食安排</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>按航班餐食安排</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>早点到机场，吃好早餐后按航班节奏休息。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix: normalize English apostrophes
</commit_message>
<xml_diff>
--- a/content/aussie-itinerary.xlsx
+++ b/content/aussie-itinerary.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="Rcaf0662ad52f4884"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="Rec59b5d3e81645a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="R41015571a2c145ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R24905560db084c24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="Ra588fa49be624df3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="R4e37d463674e4a69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="Rd9fce5cbf2794b07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R7115d181bbcc4db3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R1c7f67636cd04c77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Days" sheetId="1" r:id="Re5e99390bdc94a2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="2" r:id="R301cc00e6f564dd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resources" sheetId="3" r:id="Rf58b383e14be4f50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="4" r:id="R4289b1b4127c422a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityCosts" sheetId="5" r:id="R02fbdc4cad9e4544"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lodging" sheetId="6" r:id="Rfa9914b0fca64ef3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bookings" sheetId="7" r:id="R07175963f04e4a25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoodMap" sheetId="8" r:id="R8f65b37b68eb4e10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LedgerSnapshot" sheetId="9" r:id="R453f66920a6f43e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1245,10 +1245,10 @@
         <x:v>145.7781</x:v>
       </x:c>
       <x:c r="H12" t="str">
-        <x:v>慢享凯恩斯：Rusty’s Market 与 Palm Cove</x:v>
+        <x:v>慢享凯恩斯：Rusty's Market 与 Palm Cove</x:v>
       </x:c>
       <x:c r="I12" t="str">
-        <x:v>上午逛 Rusty’s Market，午后休整，傍晚去 Palm Cove 看海。</x:v>
+        <x:v>上午逛 Rusty's Market，午后休整，傍晚去 Palm Cove 看海。</x:v>
       </x:c>
       <x:c r="J12" t="str">
         <x:v>Southern Cross Atrium Apartments</x:v>
@@ -1481,10 +1481,10 @@
         <x:v>151.2093</x:v>
       </x:c>
       <x:c r="H16" t="str">
-        <x:v>动物园到海岸：Taronga、Bondi 与 Totti’s</x:v>
+        <x:v>动物园到海岸：Taronga、Bondi 与 Totti's</x:v>
       </x:c>
       <x:c r="I16" t="str">
-        <x:v>搭渡轮看 Taronga 的澳洲动物，下午走 Bondi 海岸，晚上在 Totti’s 用餐。</x:v>
+        <x:v>搭渡轮看 Taronga 的澳洲动物，下午走 Bondi 海岸，晚上在 Totti's 用餐。</x:v>
       </x:c>
       <x:c r="J16" t="str">
         <x:v>Oaks Sydney Goldsbrough Suites</x:v>
@@ -1505,7 +1505,7 @@
         <x:v>F2 Ferry + 打车 / 市内交通 + 步行</x:v>
       </x:c>
       <x:c r="P16" t="str">
-        <x:v>08:30–09:00 出门前往 Circular Quay；18:15 前抵达 Totti’s</x:v>
+        <x:v>08:30–09:00 出门前往 Circular Quay；18:15 前抵达 Totti's</x:v>
       </x:c>
       <x:c r="Q16" t="str">
         <x:v>oaks-sydney-map</x:v>
@@ -2393,7 +2393,7 @@
         <x:v>中午前后</x:v>
       </x:c>
       <x:c r="D29" t="str">
-        <x:v>Teddy’s Lookout</x:v>
+        <x:v>Teddy's Lookout</x:v>
       </x:c>
       <x:c r="E29" t="str">
         <x:v>S型海岸 + 河口入海</x:v>
@@ -2552,7 +2552,7 @@
         <x:v>Apollo Bay</x:v>
       </x:c>
       <x:c r="E35" t="str">
-        <x:v>Fishermen’s Co-op / seafood café 晚餐</x:v>
+        <x:v>Fishermen's Co-op / seafood café 晚餐</x:v>
       </x:c>
       <x:c r="F35" t="str">
         <x:v>海边渔港氛围</x:v>
@@ -2578,7 +2578,7 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E36" t="str">
-        <x:v>早餐：出发咖啡；午餐：Lorne café / Snow Monkey Ramen（备选）；晚餐：Apollo Bay Fishermen’s Co-op / seafood café</x:v>
+        <x:v>早餐：出发咖啡；午餐：Lorne café / Snow Monkey Ramen（备选）；晚餐：Apollo Bay Fishermen's Co-op / seafood café</x:v>
       </x:c>
       <x:c r="F36" t="str">
         <x:v>当天餐食节奏</x:v>
@@ -3302,7 +3302,7 @@
         <x:v>码头附近</x:v>
       </x:c>
       <x:c r="E64" t="str">
-        <x:v>Prawn Star / Salt House / Dundee’s 可选</x:v>
+        <x:v>Prawn Star / Salt House / Dundee's 可选</x:v>
       </x:c>
       <x:c r="F64" t="str">
         <x:v>海边晚餐</x:v>
@@ -3757,10 +3757,10 @@
         <x:v>上午</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>Rusty’s Market 买热带水果、咖啡、简单早餐</x:v>
+        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>Rusty’s Market 买热带水果、咖啡、简单早餐</x:v>
+        <x:v>Rusty's Market 买热带水果、咖啡、简单早餐</x:v>
       </x:c>
       <x:c r="F82" t="str">
         <x:v>周五正好开市，适合补水果和轻食</x:v>
@@ -3888,7 +3888,7 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>早餐：Rusty’s Market / Market水果；午餐：简餐；晚餐：Prawn Star / seafood café（优先）</x:v>
+        <x:v>早餐：Rusty's Market / Market水果；午餐：简餐；晚餐：Prawn Star / seafood café（优先）</x:v>
       </x:c>
       <x:c r="F87" t="str">
         <x:v>当天餐食节奏</x:v>
@@ -4146,7 +4146,7 @@
         <x:v>Opera House 外观</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>歌剧院外观、台阶、Man O’War Steps 初拍</x:v>
+        <x:v>歌剧院外观、台阶、Man O'War Steps 初拍</x:v>
       </x:c>
       <x:c r="F97" t="str">
         <x:v>悉尼核心地标</x:v>
@@ -4282,7 +4282,7 @@
         <x:v>海港景观非常好</x:v>
       </x:c>
       <x:c r="G102" t="str">
-        <x:v>沿海港步道慢慢走向 Mrs Macquarie’s Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
+        <x:v>沿海港步道慢慢走向 Mrs Macquarie's Chair，途中可从草坪远望歌剧院与海港桥。</x:v>
       </x:c>
       <x:c r="H102" t="str">
         <x:v>botanic-garden-map</x:v>
@@ -4299,7 +4299,7 @@
         <x:v>14:10–15:10</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Mrs Macquarie’s Chair</x:v>
+        <x:v>Mrs Macquarie's Chair</x:v>
       </x:c>
       <x:c r="E103" t="str">
         <x:v>歌剧院 + 海港大桥同框</x:v>
@@ -4380,7 +4380,7 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>早餐：bills / Toby’s Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
+        <x:v>早餐：bills / Toby's Estate；午餐：The Rocks Markets / Circular Quay 简餐；晚餐：Hello Auntie</x:v>
       </x:c>
       <x:c r="F106" t="str">
         <x:v>当天餐食节奏</x:v>
@@ -4845,7 +4845,7 @@
         <x:v>18:30</x:v>
       </x:c>
       <x:c r="D124" t="str">
-        <x:v>Totti’s Bondi</x:v>
+        <x:v>Totti's Bondi</x:v>
       </x:c>
       <x:c r="E124" t="str">
         <x:v>分享式 Italian 晚餐（已订）</x:v>
@@ -4874,13 +4874,13 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E125" t="str">
-        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti’s Bondi 18:30（已订）</x:v>
+        <x:v>早餐：CBD café；午餐：Taronga Zoo 轻食 / Circular Quay 简餐；晚餐：Totti's Bondi 18:30（已订）</x:v>
       </x:c>
       <x:c r="F125" t="str">
         <x:v>当天餐食节奏</x:v>
       </x:c>
       <x:c r="G125" t="str">
-        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti’s。</x:v>
+        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
       </x:c>
       <x:c r="H125" t="str">
         <x:v>taronga-zoo-map,circular-quay-map,bondi-map,tottis-bondi-map,tottis-bondi-official</x:v>
@@ -5108,7 +5108,7 @@
         <x:v>饮食安排</x:v>
       </x:c>
       <x:c r="E134" t="str">
-        <x:v>早餐：café / Single O / Toby’s Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
+        <x:v>早餐：café / Single O / Toby's Estate；午餐：若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐；晚餐：Cafe Sydney 17:30 Outdoor Terrace Dining（已订）</x:v>
       </x:c>
       <x:c r="F134" t="str">
         <x:v>当天餐食节奏</x:v>
@@ -6584,7 +6584,7 @@
         <x:v>fishermens-coop-map</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>Apollo Bay Fishermen’s Co-op</x:v>
+        <x:v>Apollo Bay Fishermen's Co-op</x:v>
       </x:c>
       <x:c r="C74" t="str">
         <x:v>restaurant</x:v>
@@ -6717,7 +6717,7 @@
         <x:v>dundees-map</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>Dundee’s Cairns</x:v>
+        <x:v>Dundee's Cairns</x:v>
       </x:c>
       <x:c r="C81" t="str">
         <x:v>restaurant</x:v>
@@ -7059,7 +7059,7 @@
         <x:v>tobys-estate-map</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>Toby’s Estate Sydney</x:v>
+        <x:v>Toby's Estate Sydney</x:v>
       </x:c>
       <x:c r="C99" t="str">
         <x:v>restaurant</x:v>
@@ -7912,10 +7912,8 @@
           <x:t xml:space="preserve">约 ¥7,500</x:t>
         </x:is>
       </x:c>
-      <x:c r="D7" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">不含 Cafe Sydney；含咖啡、brunch、pub、海鲜、Totti’s Bondi、夜市、超市补给、D4 BBQ-style 食材等</x:t>
-        </x:is>
+      <x:c r="D7" s="28" t="str">
+        <x:v>不含 Cafe Sydney；含咖啡、brunch、pub、海鲜、Totti's Bondi、夜市、超市补给、D4 BBQ-style 食材等</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -8859,10 +8857,8 @@
           <x:t xml:space="preserve">餐饮点多数不提前锁死。</x:t>
         </x:is>
       </x:c>
-      <x:c r="E6" s="28" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Prawn Star 可看是否需要订位；Hello Auntie 为 D12 晚餐备选；Sydney Fish Market 自由活动；Icebergs / Bondi Bistro 因 Totti’s 已订降级为备选；Lune Croissanterie 看排队和路线。</x:t>
-        </x:is>
+      <x:c r="E6" s="28" t="str">
+        <x:v>Prawn Star 可看是否需要订位；Hello Auntie 为 D12 晚餐备选；Sydney Fish Market 自由活动；Icebergs / Bondi Bistro 因 Totti's 已订降级为备选；Lune Croissanterie 看排队和路线。</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -8988,7 +8984,7 @@
         <x:v>Lorne café / Snow Monkey Ramen（备选）</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>Apollo Bay Fishermen’s Co-op / seafood café</x:v>
+        <x:v>Apollo Bay Fishermen's Co-op / seafood café</x:v>
       </x:c>
       <x:c r="E4" t="str">
         <x:v>海岸驾驶日以轻松好吃为主，Apollo Bay 的 fish &amp; chips / 海鲜正合适。</x:v>
@@ -9101,7 +9097,7 @@
         <x:v>D10 凯恩斯</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Rusty’s Market / Market水果</x:v>
+        <x:v>Rusty's Market / Market水果</x:v>
       </x:c>
       <x:c r="C11" t="str">
         <x:v>简餐</x:v>
@@ -9135,7 +9131,7 @@
         <x:v>D12 悉尼</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>bills / Toby’s Estate</x:v>
+        <x:v>bills / Toby's Estate</x:v>
       </x:c>
       <x:c r="C13" t="str">
         <x:v>The Rocks Markets / Circular Quay 简餐</x:v>
@@ -9175,10 +9171,10 @@
         <x:v>Taronga Zoo 轻食 / Circular Quay 简餐</x:v>
       </x:c>
       <x:c r="D15" t="str">
-        <x:v>Totti’s Bondi 18:30（已订）</x:v>
+        <x:v>Totti's Bondi 18:30（已订）</x:v>
       </x:c>
       <x:c r="E15" t="str">
-        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti’s。</x:v>
+        <x:v>动物园午餐简单些，海边散步结束后从容前往 18:30 的 Totti's。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" s="23" customFormat="1" ht="40" customHeight="1">
@@ -9186,7 +9182,7 @@
         <x:v>D15 Manly 弹性 + 告别</x:v>
       </x:c>
       <x:c r="B16" s="25" t="str">
-        <x:v>café / Single O / Toby’s Estate</x:v>
+        <x:v>café / Single O / Toby's Estate</x:v>
       </x:c>
       <x:c r="C16" s="25" t="str">
         <x:v>若去 Manly 则 fish &amp; chips / café，否则 CBD 简餐</x:v>

</xml_diff>